<commit_message>
slight changes, redis impl
</commit_message>
<xml_diff>
--- a/lottopy_site/lottopy/lottopy_web_edition/cash25.xlsx
+++ b/lottopy_site/lottopy/lottopy_web_edition/cash25.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C209"/>
+  <dimension ref="A1:C210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,12 +446,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>05/20/2022</t>
+          <t>05/27/2022</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>4–9–15–18–23–25</t>
+          <t>3–6–8–13–24–25</t>
         </is>
       </c>
     </row>
@@ -461,12 +461,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>05/19/2022</t>
+          <t>05/26/2022</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>4–7–9–10–14–16</t>
+          <t>1–2–4–7–15–18</t>
         </is>
       </c>
     </row>
@@ -476,12 +476,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>05/17/2022</t>
+          <t>05/24/2022</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1–6–12–13–16–25</t>
+          <t>2–4–9–13–16–22</t>
         </is>
       </c>
     </row>
@@ -491,12 +491,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>05/16/2022</t>
+          <t>05/23/2022</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5–6–8–20–22–25</t>
+          <t>5–6–7–11–14–21</t>
         </is>
       </c>
     </row>
@@ -506,12 +506,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05/13/2022</t>
+          <t>05/20/2022</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2–9–10–12–13–16</t>
+          <t>4–9–15–18–23–25</t>
         </is>
       </c>
     </row>
@@ -521,12 +521,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05/12/2022</t>
+          <t>05/19/2022</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2–4–13–15–18–25</t>
+          <t>4–7–9–10–14–16</t>
         </is>
       </c>
     </row>
@@ -536,12 +536,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05/10/2022</t>
+          <t>05/17/2022</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2–6–17–19–21–23</t>
+          <t>1–6–12–13–16–25</t>
         </is>
       </c>
     </row>
@@ -551,12 +551,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05/09/2022</t>
+          <t>05/16/2022</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>3–5–10–13–18–20</t>
+          <t>5–6–8–20–22–25</t>
         </is>
       </c>
     </row>
@@ -566,12 +566,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05/06/2022</t>
+          <t>05/13/2022</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>3–7–13–14–24–25</t>
+          <t>2–9–10–12–13–16</t>
         </is>
       </c>
     </row>
@@ -581,12 +581,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05/05/2022</t>
+          <t>05/12/2022</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>3–5–8–17–18–25</t>
+          <t>2–4–13–15–18–25</t>
         </is>
       </c>
     </row>
@@ -596,12 +596,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>05/03/2022</t>
+          <t>05/10/2022</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1–4–13–20–22–25</t>
+          <t>2–6–17–19–21–23</t>
         </is>
       </c>
     </row>
@@ -611,12 +611,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>05/02/2022</t>
+          <t>05/09/2022</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3–8–17–20–22–25</t>
+          <t>3–5–10–13–18–20</t>
         </is>
       </c>
     </row>
@@ -626,12 +626,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>04/29/2022</t>
+          <t>05/06/2022</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5–6–12–17–18–23</t>
+          <t>3–7–13–14–24–25</t>
         </is>
       </c>
     </row>
@@ -641,12 +641,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>04/28/2022</t>
+          <t>05/05/2022</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1–5–10–19–20–23</t>
+          <t>3–5–8–17–18–25</t>
         </is>
       </c>
     </row>
@@ -656,12 +656,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>04/26/2022</t>
+          <t>05/03/2022</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1–4–9–15–19–22</t>
+          <t>1–4–13–20–22–25</t>
         </is>
       </c>
     </row>
@@ -671,12 +671,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>04/25/2022</t>
+          <t>05/02/2022</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1–2–9–18–23–24</t>
+          <t>3–8–17–20–22–25</t>
         </is>
       </c>
     </row>
@@ -686,12 +686,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>04/22/2022</t>
+          <t>04/29/2022</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1–8–16–17–19–22</t>
+          <t>5–6–12–17–18–23</t>
         </is>
       </c>
     </row>
@@ -701,12 +701,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>04/21/2022</t>
+          <t>04/28/2022</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>3–11–19–22–23–24</t>
+          <t>1–5–10–19–20–23</t>
         </is>
       </c>
     </row>
@@ -716,12 +716,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>04/19/2022</t>
+          <t>04/26/2022</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>7–8–9–10–16–23</t>
+          <t>1–4–9–15–19–22</t>
         </is>
       </c>
     </row>
@@ -731,12 +731,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>04/18/2022</t>
+          <t>04/25/2022</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1–18–20–21–22–23</t>
+          <t>1–2–9–18–23–24</t>
         </is>
       </c>
     </row>
@@ -746,12 +746,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>04/15/2022</t>
+          <t>04/22/2022</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2–11–14–17–22–23</t>
+          <t>1–8–16–17–19–22</t>
         </is>
       </c>
     </row>
@@ -761,12 +761,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>04/14/2022</t>
+          <t>04/21/2022</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2–3–5–11–21–23</t>
+          <t>3–11–19–22–23–24</t>
         </is>
       </c>
     </row>
@@ -776,12 +776,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>04/12/2022</t>
+          <t>04/19/2022</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1–6–14–17–19–23</t>
+          <t>7–8–9–10–16–23</t>
         </is>
       </c>
     </row>
@@ -791,12 +791,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>04/11/2022</t>
+          <t>04/18/2022</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>12–13–14–19–21–22</t>
+          <t>1–18–20–21–22–23</t>
         </is>
       </c>
     </row>
@@ -806,12 +806,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>04/08/2022</t>
+          <t>04/15/2022</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>1–2–6–13–15–21</t>
+          <t>2–11–14–17–22–23</t>
         </is>
       </c>
     </row>
@@ -821,12 +821,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>04/07/2022</t>
+          <t>04/14/2022</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>5–10–11–12–14–15</t>
+          <t>2–3–5–11–21–23</t>
         </is>
       </c>
     </row>
@@ -836,12 +836,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>04/05/2022</t>
+          <t>04/12/2022</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2–4–6–13–14–23</t>
+          <t>1–6–14–17–19–23</t>
         </is>
       </c>
     </row>
@@ -851,12 +851,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>04/04/2022</t>
+          <t>04/11/2022</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>5–11–14–15–16–17</t>
+          <t>12–13–14–19–21–22</t>
         </is>
       </c>
     </row>
@@ -866,12 +866,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>04/01/2022</t>
+          <t>04/08/2022</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2–9–16–19–20–21</t>
+          <t>1–2–6–13–15–21</t>
         </is>
       </c>
     </row>
@@ -881,12 +881,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>03/31/2022</t>
+          <t>04/07/2022</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>5–11–13–14–18–22</t>
+          <t>5–10–11–12–14–15</t>
         </is>
       </c>
     </row>
@@ -896,12 +896,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>03/29/2022</t>
+          <t>04/05/2022</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2–4–9–16–18–19</t>
+          <t>2–4–6–13–14–23</t>
         </is>
       </c>
     </row>
@@ -911,12 +911,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>03/28/2022</t>
+          <t>04/04/2022</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>5–9–10–15–21–22</t>
+          <t>5–11–14–15–16–17</t>
         </is>
       </c>
     </row>
@@ -926,12 +926,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>03/25/2022</t>
+          <t>04/01/2022</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>6–7–16–18–23–25</t>
+          <t>2–9–16–19–20–21</t>
         </is>
       </c>
     </row>
@@ -941,12 +941,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>03/24/2022</t>
+          <t>03/31/2022</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>5–9–15–16–17–21</t>
+          <t>5–11–13–14–18–22</t>
         </is>
       </c>
     </row>
@@ -956,12 +956,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>03/22/2022</t>
+          <t>03/29/2022</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2–6–10–11–16–23</t>
+          <t>2–4–9–16–18–19</t>
         </is>
       </c>
     </row>
@@ -971,12 +971,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>03/21/2022</t>
+          <t>03/28/2022</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>6–9–14–16–22–23</t>
+          <t>5–9–10–15–21–22</t>
         </is>
       </c>
     </row>
@@ -986,12 +986,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>03/18/2022</t>
+          <t>03/25/2022</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>1–4–19–20–23–25</t>
+          <t>6–7–16–18–23–25</t>
         </is>
       </c>
     </row>
@@ -1001,12 +1001,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>03/17/2022</t>
+          <t>03/24/2022</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>1–3–4–5–8–16</t>
+          <t>5–9–15–16–17–21</t>
         </is>
       </c>
     </row>
@@ -1016,12 +1016,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>03/15/2022</t>
+          <t>03/22/2022</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>5–9–16–17–19–21</t>
+          <t>2–6–10–11–16–23</t>
         </is>
       </c>
     </row>
@@ -1031,12 +1031,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>03/14/2022</t>
+          <t>03/21/2022</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>1–4–7–13–16–24</t>
+          <t>6–9–14–16–22–23</t>
         </is>
       </c>
     </row>
@@ -1046,12 +1046,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>03/11/2022</t>
+          <t>03/18/2022</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>6–13–15–18–21–23</t>
+          <t>1–4–19–20–23–25</t>
         </is>
       </c>
     </row>
@@ -1061,12 +1061,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>03/10/2022</t>
+          <t>03/17/2022</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2–4–15–16–19–21</t>
+          <t>1–3–4–5–8–16</t>
         </is>
       </c>
     </row>
@@ -1076,12 +1076,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>03/08/2022</t>
+          <t>03/15/2022</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>1–3–4–7–10–20</t>
+          <t>5–9–16–17–19–21</t>
         </is>
       </c>
     </row>
@@ -1091,12 +1091,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>03/07/2022</t>
+          <t>03/14/2022</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>1–4–8–15–24–25</t>
+          <t>1–4–7–13–16–24</t>
         </is>
       </c>
     </row>
@@ -1106,12 +1106,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>03/04/2022</t>
+          <t>03/11/2022</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2–5–9–12–18–24</t>
+          <t>6–13–15–18–21–23</t>
         </is>
       </c>
     </row>
@@ -1121,12 +1121,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>03/03/2022</t>
+          <t>03/10/2022</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>6–7–9–12–14–22</t>
+          <t>2–4–15–16–19–21</t>
         </is>
       </c>
     </row>
@@ -1136,12 +1136,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>03/01/2022</t>
+          <t>03/08/2022</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2–7–9–14–16–20</t>
+          <t>1–3–4–7–10–20</t>
         </is>
       </c>
     </row>
@@ -1151,12 +1151,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>02/28/2022</t>
+          <t>03/07/2022</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>1–6–7–19–22–24</t>
+          <t>1–4–8–15–24–25</t>
         </is>
       </c>
     </row>
@@ -1166,12 +1166,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>02/25/2022</t>
+          <t>03/04/2022</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>3–7–9–14–15–22</t>
+          <t>2–5–9–12–18–24</t>
         </is>
       </c>
     </row>
@@ -1181,12 +1181,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>02/24/2022</t>
+          <t>03/03/2022</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>5–13–14–15–22–24</t>
+          <t>6–7–9–12–14–22</t>
         </is>
       </c>
     </row>
@@ -1196,12 +1196,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>02/22/2022</t>
+          <t>03/01/2022</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>6–9–18–20–22–23</t>
+          <t>2–7–9–14–16–20</t>
         </is>
       </c>
     </row>
@@ -1211,12 +1211,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>02/21/2022</t>
+          <t>02/28/2022</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>3–11–15–16–17–21</t>
+          <t>1–6–7–19–22–24</t>
         </is>
       </c>
     </row>
@@ -1226,12 +1226,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>02/18/2022</t>
+          <t>02/25/2022</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>1–2–10–14–22–23</t>
+          <t>3–7–9–14–15–22</t>
         </is>
       </c>
     </row>
@@ -1241,12 +1241,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>02/17/2022</t>
+          <t>02/24/2022</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>3–4–10–19–22–24</t>
+          <t>5–13–14–15–22–24</t>
         </is>
       </c>
     </row>
@@ -1256,12 +1256,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>02/15/2022</t>
+          <t>02/22/2022</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>1–9–13–15–19–20</t>
+          <t>6–9–18–20–22–23</t>
         </is>
       </c>
     </row>
@@ -1271,12 +1271,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>02/14/2022</t>
+          <t>02/21/2022</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>4–7–9–10–14–17</t>
+          <t>3–11–15–16–17–21</t>
         </is>
       </c>
     </row>
@@ -1286,12 +1286,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>02/11/2022</t>
+          <t>02/18/2022</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>4–6–8–10–12–20</t>
+          <t>1–2–10–14–22–23</t>
         </is>
       </c>
     </row>
@@ -1301,12 +1301,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>02/10/2022</t>
+          <t>02/17/2022</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>5–11–16–20–22–23</t>
+          <t>3–4–10–19–22–24</t>
         </is>
       </c>
     </row>
@@ -1316,12 +1316,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>02/08/2022</t>
+          <t>02/15/2022</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2–5–14–16–17–25</t>
+          <t>1–9–13–15–19–20</t>
         </is>
       </c>
     </row>
@@ -1331,12 +1331,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>02/07/2022</t>
+          <t>02/14/2022</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>4–7–14–16–18–23</t>
+          <t>4–7–9–10–14–17</t>
         </is>
       </c>
     </row>
@@ -1346,12 +1346,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>02/04/2022</t>
+          <t>02/11/2022</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>13–17–20–23–24–25</t>
+          <t>4–6–8–10–12–20</t>
         </is>
       </c>
     </row>
@@ -1361,12 +1361,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>02/03/2022</t>
+          <t>02/10/2022</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>6–12–14–17–22–25</t>
+          <t>5–11–16–20–22–23</t>
         </is>
       </c>
     </row>
@@ -1376,12 +1376,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>02/01/2022</t>
+          <t>02/08/2022</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>6–7–12–15–16–20</t>
+          <t>2–5–14–16–17–25</t>
         </is>
       </c>
     </row>
@@ -1391,12 +1391,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>01/31/2022</t>
+          <t>02/07/2022</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>5–7–8–9–10–22</t>
+          <t>4–7–14–16–18–23</t>
         </is>
       </c>
     </row>
@@ -1406,12 +1406,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>01/28/2022</t>
+          <t>02/04/2022</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>7–9–11–12–17–19</t>
+          <t>13–17–20–23–24–25</t>
         </is>
       </c>
     </row>
@@ -1421,12 +1421,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>01/27/2022</t>
+          <t>02/03/2022</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2–3–14–19–20–21</t>
+          <t>6–12–14–17–22–25</t>
         </is>
       </c>
     </row>
@@ -1436,12 +1436,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>01/25/2022</t>
+          <t>02/01/2022</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>3–4–5–11–17–19</t>
+          <t>6–7–12–15–16–20</t>
         </is>
       </c>
     </row>
@@ -1451,12 +1451,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>01/24/2022</t>
+          <t>01/31/2022</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>4–7–8–20–21–25</t>
+          <t>5–7–8–9–10–22</t>
         </is>
       </c>
     </row>
@@ -1466,12 +1466,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>01/21/2022</t>
+          <t>01/28/2022</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>8–11–14–15–18–24</t>
+          <t>7–9–11–12–17–19</t>
         </is>
       </c>
     </row>
@@ -1481,12 +1481,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>01/20/2022</t>
+          <t>01/27/2022</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2–15–19–20–22–24</t>
+          <t>2–3–14–19–20–21</t>
         </is>
       </c>
     </row>
@@ -1496,12 +1496,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>01/18/2022</t>
+          <t>01/25/2022</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>3–5–16–17–18–21</t>
+          <t>3–4–5–11–17–19</t>
         </is>
       </c>
     </row>
@@ -1511,12 +1511,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>01/17/2022</t>
+          <t>01/24/2022</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>5–8–16–18–20–22</t>
+          <t>4–7–8–20–21–25</t>
         </is>
       </c>
     </row>
@@ -1526,12 +1526,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>01/14/2022</t>
+          <t>01/21/2022</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2–5–8–9–10–13</t>
+          <t>8–11–14–15–18–24</t>
         </is>
       </c>
     </row>
@@ -1541,12 +1541,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>01/13/2022</t>
+          <t>01/20/2022</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2–6–8–11–18–21</t>
+          <t>2–15–19–20–22–24</t>
         </is>
       </c>
     </row>
@@ -1556,12 +1556,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>01/11/2022</t>
+          <t>01/18/2022</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>7–8–9–15–19–23</t>
+          <t>3–5–16–17–18–21</t>
         </is>
       </c>
     </row>
@@ -1571,12 +1571,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>01/10/2022</t>
+          <t>01/17/2022</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>10–13–14–19–22–23</t>
+          <t>5–8–16–18–20–22</t>
         </is>
       </c>
     </row>
@@ -1586,12 +1586,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>01/07/2022</t>
+          <t>01/14/2022</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>4–8–21–23–24–25</t>
+          <t>2–5–8–9–10–13</t>
         </is>
       </c>
     </row>
@@ -1601,12 +1601,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>01/06/2022</t>
+          <t>01/13/2022</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>7–9–10–17–18–23</t>
+          <t>2–6–8–11–18–21</t>
         </is>
       </c>
     </row>
@@ -1616,12 +1616,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>01/04/2022</t>
+          <t>01/11/2022</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>4–7–14–15–24–25</t>
+          <t>7–8–9–15–19–23</t>
         </is>
       </c>
     </row>
@@ -1631,12 +1631,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>01/03/2022</t>
+          <t>01/10/2022</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>6–10–17–18–19–21</t>
+          <t>10–13–14–19–22–23</t>
         </is>
       </c>
     </row>
@@ -1646,12 +1646,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>12/31/2021</t>
+          <t>01/07/2022</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>11–17–20–22–23–24</t>
+          <t>4–8–21–23–24–25</t>
         </is>
       </c>
     </row>
@@ -1661,12 +1661,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>12/30/2021</t>
+          <t>01/06/2022</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>1–8–9–13–20–25</t>
+          <t>7–9–10–17–18–23</t>
         </is>
       </c>
     </row>
@@ -1676,12 +1676,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>12/28/2021</t>
+          <t>01/04/2022</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>4–9–11–15–16–25</t>
+          <t>4–7–14–15–24–25</t>
         </is>
       </c>
     </row>
@@ -1691,12 +1691,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>12/27/2021</t>
+          <t>01/03/2022</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>3–4–10–14–19–25</t>
+          <t>6–10–17–18–19–21</t>
         </is>
       </c>
     </row>
@@ -1706,12 +1706,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>12/24/2021</t>
+          <t>12/31/2021</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>4–6–13–17–21–22</t>
+          <t>11–17–20–22–23–24</t>
         </is>
       </c>
     </row>
@@ -1721,12 +1721,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>12/23/2021</t>
+          <t>12/30/2021</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>1–2–3–15–20–23</t>
+          <t>1–8–9–13–20–25</t>
         </is>
       </c>
     </row>
@@ -1736,12 +1736,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>12/21/2021</t>
+          <t>12/28/2021</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>6–9–11–12–14–25</t>
+          <t>4–9–11–15–16–25</t>
         </is>
       </c>
     </row>
@@ -1751,12 +1751,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>12/20/2021</t>
+          <t>12/27/2021</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>7–8–9–22–23–24</t>
+          <t>3–4–10–14–19–25</t>
         </is>
       </c>
     </row>
@@ -1766,12 +1766,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>12/17/2021</t>
+          <t>12/24/2021</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>3–9–15–16–18–22</t>
+          <t>4–6–13–17–21–22</t>
         </is>
       </c>
     </row>
@@ -1781,12 +1781,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>12/16/2021</t>
+          <t>12/23/2021</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2–3–11–13–24–25</t>
+          <t>1–2–3–15–20–23</t>
         </is>
       </c>
     </row>
@@ -1796,12 +1796,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>12/14/2021</t>
+          <t>12/21/2021</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2–7–9–17–23–24</t>
+          <t>6–9–11–12–14–25</t>
         </is>
       </c>
     </row>
@@ -1811,12 +1811,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>12/13/2021</t>
+          <t>12/20/2021</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2–6–15–16–23–24</t>
+          <t>7–8–9–22–23–24</t>
         </is>
       </c>
     </row>
@@ -1826,12 +1826,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>12/10/2021</t>
+          <t>12/17/2021</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>3–6–9–10–14–21</t>
+          <t>3–9–15–16–18–22</t>
         </is>
       </c>
     </row>
@@ -1841,12 +1841,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>12/09/2021</t>
+          <t>12/16/2021</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2–12–14–15–19–21</t>
+          <t>2–3–11–13–24–25</t>
         </is>
       </c>
     </row>
@@ -1856,12 +1856,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>12/07/2021</t>
+          <t>12/14/2021</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>3–5–8–9–16–25</t>
+          <t>2–7–9–17–23–24</t>
         </is>
       </c>
     </row>
@@ -1871,12 +1871,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>12/06/2021</t>
+          <t>12/13/2021</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>3–5–8–12–15–19</t>
+          <t>2–6–15–16–23–24</t>
         </is>
       </c>
     </row>
@@ -1886,12 +1886,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>12/03/2021</t>
+          <t>12/10/2021</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>10–13–14–15–21–24</t>
+          <t>3–6–9–10–14–21</t>
         </is>
       </c>
     </row>
@@ -1901,12 +1901,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>12/02/2021</t>
+          <t>12/09/2021</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2–7–8–11–22–24</t>
+          <t>2–12–14–15–19–21</t>
         </is>
       </c>
     </row>
@@ -1916,12 +1916,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>11/30/2021</t>
+          <t>12/07/2021</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>12–14–20–23–24–25</t>
+          <t>3–5–8–9–16–25</t>
         </is>
       </c>
     </row>
@@ -1931,12 +1931,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>11/29/2021</t>
+          <t>12/06/2021</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>4–8–10–13–20–21</t>
+          <t>3–5–8–12–15–19</t>
         </is>
       </c>
     </row>
@@ -1946,12 +1946,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>11/26/2021</t>
+          <t>12/03/2021</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>3–7–14–17–24–25</t>
+          <t>10–13–14–15–21–24</t>
         </is>
       </c>
     </row>
@@ -1961,12 +1961,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>11/25/2021</t>
+          <t>12/02/2021</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2–11–16–18–20–21</t>
+          <t>2–7–8–11–22–24</t>
         </is>
       </c>
     </row>
@@ -1976,12 +1976,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>11/23/2021</t>
+          <t>11/30/2021</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2–10–11–12–14–19</t>
+          <t>12–14–20–23–24–25</t>
         </is>
       </c>
     </row>
@@ -1991,12 +1991,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>11/22/2021</t>
+          <t>11/29/2021</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>5–10–12–16–20–25</t>
+          <t>4–8–10–13–20–21</t>
         </is>
       </c>
     </row>
@@ -2006,12 +2006,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>11/19/2021</t>
+          <t>11/26/2021</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>12–16–19–20–21–24</t>
+          <t>3–7–14–17–24–25</t>
         </is>
       </c>
     </row>
@@ -2021,12 +2021,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>11/18/2021</t>
+          <t>11/25/2021</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>1–4–17–18–20–23</t>
+          <t>2–11–16–18–20–21</t>
         </is>
       </c>
     </row>
@@ -2036,12 +2036,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>11/16/2021</t>
+          <t>11/23/2021</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>5–8–10–11–16–23</t>
+          <t>2–10–11–12–14–19</t>
         </is>
       </c>
     </row>
@@ -2051,12 +2051,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>11/15/2021</t>
+          <t>11/22/2021</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2–6–10–11–15–18</t>
+          <t>5–10–12–16–20–25</t>
         </is>
       </c>
     </row>
@@ -2066,12 +2066,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>11/12/2021</t>
+          <t>11/19/2021</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>1–13–14–15–22–25</t>
+          <t>12–16–19–20–21–24</t>
         </is>
       </c>
     </row>
@@ -2081,12 +2081,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>11/11/2021</t>
+          <t>11/18/2021</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2–3–5–14–21–22</t>
+          <t>1–4–17–18–20–23</t>
         </is>
       </c>
     </row>
@@ -2096,12 +2096,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>11/09/2021</t>
+          <t>11/16/2021</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2–4–10–13–16–23</t>
+          <t>5–8–10–11–16–23</t>
         </is>
       </c>
     </row>
@@ -2111,12 +2111,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>11/08/2021</t>
+          <t>11/15/2021</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>1–2–8–10–13–24</t>
+          <t>2–6–10–11–15–18</t>
         </is>
       </c>
     </row>
@@ -2126,12 +2126,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>11/05/2021</t>
+          <t>11/12/2021</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>4–11–12–18–19–25</t>
+          <t>1–13–14–15–22–25</t>
         </is>
       </c>
     </row>
@@ -2141,12 +2141,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>11/04/2021</t>
+          <t>11/11/2021</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>10–15–19–21–24–25</t>
+          <t>2–3–5–14–21–22</t>
         </is>
       </c>
     </row>
@@ -2156,12 +2156,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>11/02/2021</t>
+          <t>11/09/2021</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>3–4–9–16–17–18</t>
+          <t>2–4–10–13–16–23</t>
         </is>
       </c>
     </row>
@@ -2171,12 +2171,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>11/01/2021</t>
+          <t>11/08/2021</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>5–6–14–15–18–20</t>
+          <t>1–2–8–10–13–24</t>
         </is>
       </c>
     </row>
@@ -2186,12 +2186,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>10/29/2021</t>
+          <t>11/05/2021</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2–3–8–9–13–15</t>
+          <t>4–11–12–18–19–25</t>
         </is>
       </c>
     </row>
@@ -2201,12 +2201,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>10/28/2021</t>
+          <t>11/04/2021</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>7–15–19–20–23–24</t>
+          <t>10–15–19–21–24–25</t>
         </is>
       </c>
     </row>
@@ -2216,12 +2216,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>10/26/2021</t>
+          <t>11/02/2021</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>3–4–14–16–17–25</t>
+          <t>3–4–9–16–17–18</t>
         </is>
       </c>
     </row>
@@ -2231,12 +2231,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>10/25/2021</t>
+          <t>11/01/2021</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>9–12–17–19–20–24</t>
+          <t>5–6–14–15–18–20</t>
         </is>
       </c>
     </row>
@@ -2246,12 +2246,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>10/22/2021</t>
+          <t>10/29/2021</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2–5–6–18–20–23</t>
+          <t>2–3–8–9–13–15</t>
         </is>
       </c>
     </row>
@@ -2261,12 +2261,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>10/21/2021</t>
+          <t>10/28/2021</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>5–8–9–13–22–24</t>
+          <t>7–15–19–20–23–24</t>
         </is>
       </c>
     </row>
@@ -2276,12 +2276,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>10/19/2021</t>
+          <t>10/26/2021</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>8–9–11–15–19–25</t>
+          <t>3–4–14–16–17–25</t>
         </is>
       </c>
     </row>
@@ -2291,12 +2291,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>10/18/2021</t>
+          <t>10/25/2021</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>3–4–8–10–12–20</t>
+          <t>9–12–17–19–20–24</t>
         </is>
       </c>
     </row>
@@ -2306,12 +2306,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>10/15/2021</t>
+          <t>10/22/2021</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>1–3–4–8–19–21</t>
+          <t>2–5–6–18–20–23</t>
         </is>
       </c>
     </row>
@@ -2321,12 +2321,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>10/14/2021</t>
+          <t>10/21/2021</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2–5–8–15–16–23</t>
+          <t>5–8–9–13–22–24</t>
         </is>
       </c>
     </row>
@@ -2336,12 +2336,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>10/12/2021</t>
+          <t>10/19/2021</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>5–6–13–14–24–25</t>
+          <t>8–9–11–15–19–25</t>
         </is>
       </c>
     </row>
@@ -2351,12 +2351,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>10/11/2021</t>
+          <t>10/18/2021</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>1–2–3–5–21–23</t>
+          <t>3–4–8–10–12–20</t>
         </is>
       </c>
     </row>
@@ -2366,12 +2366,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>10/08/2021</t>
+          <t>10/15/2021</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>10–11–13–17–20–22</t>
+          <t>1–3–4–8–19–21</t>
         </is>
       </c>
     </row>
@@ -2381,12 +2381,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>10/07/2021</t>
+          <t>10/14/2021</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>3–5–8–16–19–23</t>
+          <t>2–5–8–15–16–23</t>
         </is>
       </c>
     </row>
@@ -2396,12 +2396,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>10/05/2021</t>
+          <t>10/12/2021</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>7–9–13–15–18–23</t>
+          <t>5–6–13–14–24–25</t>
         </is>
       </c>
     </row>
@@ -2411,12 +2411,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>10/04/2021</t>
+          <t>10/11/2021</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>8–9–11–18–20–23</t>
+          <t>1–2–3–5–21–23</t>
         </is>
       </c>
     </row>
@@ -2426,12 +2426,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>10/01/2021</t>
+          <t>10/08/2021</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2–3–5–7–11–18</t>
+          <t>10–11–13–17–20–22</t>
         </is>
       </c>
     </row>
@@ -2441,12 +2441,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>09/30/2021</t>
+          <t>10/07/2021</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>5–16–18–20–22–24</t>
+          <t>3–5–8–16–19–23</t>
         </is>
       </c>
     </row>
@@ -2456,12 +2456,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>09/28/2021</t>
+          <t>10/05/2021</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>1–9–11–12–18–22</t>
+          <t>7–9–13–15–18–23</t>
         </is>
       </c>
     </row>
@@ -2471,12 +2471,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>09/27/2021</t>
+          <t>10/04/2021</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>4–5–6–10–14–22</t>
+          <t>8–9–11–18–20–23</t>
         </is>
       </c>
     </row>
@@ -2486,12 +2486,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>09/24/2021</t>
+          <t>10/01/2021</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>4–11–15–16–22–25</t>
+          <t>2–3–5–7–11–18</t>
         </is>
       </c>
     </row>
@@ -2501,12 +2501,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>09/23/2021</t>
+          <t>09/30/2021</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>4–9–13–15–17–18</t>
+          <t>5–16–18–20–22–24</t>
         </is>
       </c>
     </row>
@@ -2516,12 +2516,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>09/21/2021</t>
+          <t>09/28/2021</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>1–13–14–21–22–24</t>
+          <t>1–9–11–12–18–22</t>
         </is>
       </c>
     </row>
@@ -2531,12 +2531,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>09/20/2021</t>
+          <t>09/27/2021</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>1–13–17–18–20–22</t>
+          <t>4–5–6–10–14–22</t>
         </is>
       </c>
     </row>
@@ -2546,12 +2546,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>09/17/2021</t>
+          <t>09/24/2021</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2–6–8–9–11–12</t>
+          <t>4–11–15–16–22–25</t>
         </is>
       </c>
     </row>
@@ -2561,12 +2561,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>09/16/2021</t>
+          <t>09/23/2021</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2–11–12–14–17–19</t>
+          <t>4–9–13–15–17–18</t>
         </is>
       </c>
     </row>
@@ -2576,12 +2576,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>09/14/2021</t>
+          <t>09/21/2021</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>4–11–18–19–20–23</t>
+          <t>1–13–14–21–22–24</t>
         </is>
       </c>
     </row>
@@ -2591,12 +2591,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>09/13/2021</t>
+          <t>09/20/2021</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>1–8–11–12–13–18</t>
+          <t>1–13–17–18–20–22</t>
         </is>
       </c>
     </row>
@@ -2606,12 +2606,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>09/10/2021</t>
+          <t>09/17/2021</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>3–4–6–8–11–16</t>
+          <t>2–6–8–9–11–12</t>
         </is>
       </c>
     </row>
@@ -2621,12 +2621,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>09/09/2021</t>
+          <t>09/16/2021</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>1–14–15–20–21–25</t>
+          <t>2–11–12–14–17–19</t>
         </is>
       </c>
     </row>
@@ -2636,12 +2636,12 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>09/07/2021</t>
+          <t>09/14/2021</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>5–7–8–9–18–21</t>
+          <t>4–11–18–19–20–23</t>
         </is>
       </c>
     </row>
@@ -2651,12 +2651,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>09/06/2021</t>
+          <t>09/13/2021</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>6–7–9–16–21–22</t>
+          <t>1–8–11–12–13–18</t>
         </is>
       </c>
     </row>
@@ -2666,12 +2666,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>09/03/2021</t>
+          <t>09/10/2021</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>1–3–11–21–22–24</t>
+          <t>3–4–6–8–11–16</t>
         </is>
       </c>
     </row>
@@ -2681,12 +2681,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>09/02/2021</t>
+          <t>09/09/2021</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>1–2–4–10–11–24</t>
+          <t>1–14–15–20–21–25</t>
         </is>
       </c>
     </row>
@@ -2696,12 +2696,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>08/31/2021</t>
+          <t>09/07/2021</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>1–8–9–15–19–21</t>
+          <t>5–7–8–9–18–21</t>
         </is>
       </c>
     </row>
@@ -2711,12 +2711,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>08/30/2021</t>
+          <t>09/06/2021</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>5–10–19–20–21–25</t>
+          <t>6–7–9–16–21–22</t>
         </is>
       </c>
     </row>
@@ -2726,12 +2726,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>08/27/2021</t>
+          <t>09/03/2021</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>1–10–15–17–18–21</t>
+          <t>1–3–11–21–22–24</t>
         </is>
       </c>
     </row>
@@ -2741,12 +2741,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>08/26/2021</t>
+          <t>09/02/2021</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>6–14–18–19–23–25</t>
+          <t>1–2–4–10–11–24</t>
         </is>
       </c>
     </row>
@@ -2756,12 +2756,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>08/24/2021</t>
+          <t>08/31/2021</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2–3–6–20–21–23</t>
+          <t>1–8–9–15–19–21</t>
         </is>
       </c>
     </row>
@@ -2771,12 +2771,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>08/23/2021</t>
+          <t>08/30/2021</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>9–11–12–14–18–23</t>
+          <t>5–10–19–20–21–25</t>
         </is>
       </c>
     </row>
@@ -2786,12 +2786,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>08/20/2021</t>
+          <t>08/27/2021</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>5–8–17–19–20–24</t>
+          <t>1–10–15–17–18–21</t>
         </is>
       </c>
     </row>
@@ -2801,12 +2801,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>08/19/2021</t>
+          <t>08/26/2021</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2–3–6–8–12–21</t>
+          <t>6–14–18–19–23–25</t>
         </is>
       </c>
     </row>
@@ -2816,12 +2816,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>08/17/2021</t>
+          <t>08/24/2021</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>7–12–15–16–20–25</t>
+          <t>2–3–6–20–21–23</t>
         </is>
       </c>
     </row>
@@ -2831,12 +2831,12 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>08/16/2021</t>
+          <t>08/23/2021</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>1–3–5–8–9–15</t>
+          <t>9–11–12–14–18–23</t>
         </is>
       </c>
     </row>
@@ -2846,12 +2846,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>08/13/2021</t>
+          <t>08/20/2021</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>1–5–10–14–18–24</t>
+          <t>5–8–17–19–20–24</t>
         </is>
       </c>
     </row>
@@ -2861,12 +2861,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>08/12/2021</t>
+          <t>08/19/2021</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>4–7–13–17–21–22</t>
+          <t>2–3–6–8–12–21</t>
         </is>
       </c>
     </row>
@@ -2876,12 +2876,12 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>08/10/2021</t>
+          <t>08/17/2021</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>4–6–9–10–15–24</t>
+          <t>7–12–15–16–20–25</t>
         </is>
       </c>
     </row>
@@ -2891,12 +2891,12 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>08/09/2021</t>
+          <t>08/16/2021</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>1–2–6–13–18–25</t>
+          <t>1–3–5–8–9–15</t>
         </is>
       </c>
     </row>
@@ -2906,12 +2906,12 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>08/06/2021</t>
+          <t>08/13/2021</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>5–8–9–14–23–24</t>
+          <t>1–5–10–14–18–24</t>
         </is>
       </c>
     </row>
@@ -2921,12 +2921,12 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>08/05/2021</t>
+          <t>08/12/2021</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2–5–6–12–14–18</t>
+          <t>4–7–13–17–21–22</t>
         </is>
       </c>
     </row>
@@ -2936,12 +2936,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>08/03/2021</t>
+          <t>08/10/2021</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2–7–17–22–24–25</t>
+          <t>4–6–9–10–15–24</t>
         </is>
       </c>
     </row>
@@ -2951,12 +2951,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>08/02/2021</t>
+          <t>08/09/2021</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>7–12–13–18–22–24</t>
+          <t>1–2–6–13–18–25</t>
         </is>
       </c>
     </row>
@@ -2966,12 +2966,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>07/30/2021</t>
+          <t>08/06/2021</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>3–4–13–22–24–25</t>
+          <t>5–8–9–14–23–24</t>
         </is>
       </c>
     </row>
@@ -2981,12 +2981,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>07/29/2021</t>
+          <t>08/05/2021</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>5–7–12–17–19–24</t>
+          <t>2–5–6–12–14–18</t>
         </is>
       </c>
     </row>
@@ -2996,12 +2996,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>07/27/2021</t>
+          <t>08/03/2021</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>1–4–16–17–18–21</t>
+          <t>2–7–17–22–24–25</t>
         </is>
       </c>
     </row>
@@ -3011,12 +3011,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>07/26/2021</t>
+          <t>08/02/2021</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>3–14–19–21–23–24</t>
+          <t>7–12–13–18–22–24</t>
         </is>
       </c>
     </row>
@@ -3026,12 +3026,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>07/23/2021</t>
+          <t>07/30/2021</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>9–12–14–16–22–25</t>
+          <t>3–4–13–22–24–25</t>
         </is>
       </c>
     </row>
@@ -3041,12 +3041,12 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>07/22/2021</t>
+          <t>07/29/2021</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2–5–6–15–16–20</t>
+          <t>5–7–12–17–19–24</t>
         </is>
       </c>
     </row>
@@ -3056,12 +3056,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>07/20/2021</t>
+          <t>07/27/2021</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>4–7–12–15–20–21</t>
+          <t>1–4–16–17–18–21</t>
         </is>
       </c>
     </row>
@@ -3071,12 +3071,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>07/19/2021</t>
+          <t>07/26/2021</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2–5–9–10–18–22</t>
+          <t>3–14–19–21–23–24</t>
         </is>
       </c>
     </row>
@@ -3086,12 +3086,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>07/16/2021</t>
+          <t>07/23/2021</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>4–8–10–11–12–21</t>
+          <t>9–12–14–16–22–25</t>
         </is>
       </c>
     </row>
@@ -3101,12 +3101,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>07/15/2021</t>
+          <t>07/22/2021</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>1–6–9–11–17–22</t>
+          <t>2–5–6–15–16–20</t>
         </is>
       </c>
     </row>
@@ -3116,12 +3116,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>07/13/2021</t>
+          <t>07/20/2021</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>4–11–14–15–17–18</t>
+          <t>4–7–12–15–20–21</t>
         </is>
       </c>
     </row>
@@ -3131,12 +3131,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>07/12/2021</t>
+          <t>07/19/2021</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>1–4–5–7–8–22</t>
+          <t>2–5–9–10–18–22</t>
         </is>
       </c>
     </row>
@@ -3146,12 +3146,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>07/09/2021</t>
+          <t>07/16/2021</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>7–13–14–16–21–22</t>
+          <t>4–8–10–11–12–21</t>
         </is>
       </c>
     </row>
@@ -3161,12 +3161,12 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>07/08/2021</t>
+          <t>07/15/2021</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>5–8–9–13–14–16</t>
+          <t>1–6–9–11–17–22</t>
         </is>
       </c>
     </row>
@@ -3176,12 +3176,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>07/06/2021</t>
+          <t>07/13/2021</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>1–18–20–21–22–25</t>
+          <t>4–11–14–15–17–18</t>
         </is>
       </c>
     </row>
@@ -3191,12 +3191,12 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>07/05/2021</t>
+          <t>07/12/2021</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>3–7–11–12–13–23</t>
+          <t>1–4–5–7–8–22</t>
         </is>
       </c>
     </row>
@@ -3206,12 +3206,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>07/02/2021</t>
+          <t>07/09/2021</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>1–4–5–8–14–20</t>
+          <t>7–13–14–16–21–22</t>
         </is>
       </c>
     </row>
@@ -3221,12 +3221,12 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>07/01/2021</t>
+          <t>07/08/2021</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>6–9–11–14–16–19</t>
+          <t>5–8–9–13–14–16</t>
         </is>
       </c>
     </row>
@@ -3236,12 +3236,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>06/29/2021</t>
+          <t>07/06/2021</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>1–5–9–10–16–20</t>
+          <t>1–18–20–21–22–25</t>
         </is>
       </c>
     </row>
@@ -3251,12 +3251,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>06/28/2021</t>
+          <t>07/05/2021</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>4–14–18–20–21–22</t>
+          <t>3–7–11–12–13–23</t>
         </is>
       </c>
     </row>
@@ -3266,12 +3266,12 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>06/25/2021</t>
+          <t>07/02/2021</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>1–3–4–7–11–18</t>
+          <t>1–4–5–8–14–20</t>
         </is>
       </c>
     </row>
@@ -3281,12 +3281,12 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>06/24/2021</t>
+          <t>07/01/2021</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>1–5–9–11–20–22</t>
+          <t>6–9–11–14–16–19</t>
         </is>
       </c>
     </row>
@@ -3296,12 +3296,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>06/22/2021</t>
+          <t>06/29/2021</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>7–9–12–18–21–23</t>
+          <t>1–5–9–10–16–20</t>
         </is>
       </c>
     </row>
@@ -3311,12 +3311,12 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>06/21/2021</t>
+          <t>06/28/2021</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>7–11–17–18–23–24</t>
+          <t>4–14–18–20–21–22</t>
         </is>
       </c>
     </row>
@@ -3326,12 +3326,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>06/18/2021</t>
+          <t>06/25/2021</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2–7–11–17–18–25</t>
+          <t>1–3–4–7–11–18</t>
         </is>
       </c>
     </row>
@@ -3341,12 +3341,12 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>06/17/2021</t>
+          <t>06/24/2021</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>3–12–17–19–24–25</t>
+          <t>1–5–9–11–20–22</t>
         </is>
       </c>
     </row>
@@ -3356,12 +3356,12 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>06/15/2021</t>
+          <t>06/22/2021</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>3–5–12–16–18–23</t>
+          <t>7–9–12–18–21–23</t>
         </is>
       </c>
     </row>
@@ -3371,12 +3371,12 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>06/14/2021</t>
+          <t>06/21/2021</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>1–5–11–12–22–23</t>
+          <t>7–11–17–18–23–24</t>
         </is>
       </c>
     </row>
@@ -3386,12 +3386,12 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>06/11/2021</t>
+          <t>06/18/2021</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2–5–10–11–24–25</t>
+          <t>2–7–11–17–18–25</t>
         </is>
       </c>
     </row>
@@ -3401,12 +3401,12 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>06/10/2021</t>
+          <t>06/17/2021</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>7–10–13–14–18–21</t>
+          <t>3–12–17–19–24–25</t>
         </is>
       </c>
     </row>
@@ -3416,12 +3416,12 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>06/08/2021</t>
+          <t>06/15/2021</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>8–9–15–16–23–25</t>
+          <t>3–5–12–16–18–23</t>
         </is>
       </c>
     </row>
@@ -3431,12 +3431,12 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>06/07/2021</t>
+          <t>06/14/2021</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>4–6–7–11–17–20</t>
+          <t>1–5–11–12–22–23</t>
         </is>
       </c>
     </row>
@@ -3446,12 +3446,12 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>06/04/2021</t>
+          <t>06/11/2021</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>1–2–9–15–18–24</t>
+          <t>2–5–10–11–24–25</t>
         </is>
       </c>
     </row>
@@ -3461,12 +3461,12 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>06/03/2021</t>
+          <t>06/10/2021</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>5–6–8–15–19–22</t>
+          <t>7–10–13–14–18–21</t>
         </is>
       </c>
     </row>
@@ -3476,12 +3476,12 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>06/01/2021</t>
+          <t>06/08/2021</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>4–7–12–14–21–22</t>
+          <t>8–9–15–16–23–25</t>
         </is>
       </c>
     </row>
@@ -3491,12 +3491,12 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>05/31/2021</t>
+          <t>06/07/2021</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>3–4–17–18–22–23</t>
+          <t>4–6–7–11–17–20</t>
         </is>
       </c>
     </row>
@@ -3506,12 +3506,12 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>05/28/2021</t>
+          <t>06/04/2021</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>1–3–7–11–12–14</t>
+          <t>1–2–9–15–18–24</t>
         </is>
       </c>
     </row>
@@ -3521,12 +3521,12 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>05/27/2021</t>
+          <t>06/03/2021</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>3–4–21–22–24–25</t>
+          <t>5–6–8–15–19–22</t>
         </is>
       </c>
     </row>
@@ -3536,12 +3536,12 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>05/25/2021</t>
+          <t>06/01/2021</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>3–10–12–20–22–24</t>
+          <t>4–7–12–14–21–22</t>
         </is>
       </c>
     </row>
@@ -3551,12 +3551,27 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>05/24/2021</t>
+          <t>05/31/2021</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>2–7–11–14–20–25</t>
+          <t>3–4–17–18–22–23</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="1" t="n">
+        <v>208</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>05/28/2021</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>1–3–7–11–12–14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Final touches before deployment, celery installed
</commit_message>
<xml_diff>
--- a/lottopy_site/lottopy/lottopy_web_edition/cash25.xlsx
+++ b/lottopy_site/lottopy/lottopy_web_edition/cash25.xlsx
@@ -446,12 +446,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>05/27/2022</t>
+          <t>06/07/2022</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>3–6–8–13–24–25</t>
+          <t>2–8–10–11–12–22</t>
         </is>
       </c>
     </row>
@@ -461,12 +461,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>05/26/2022</t>
+          <t>06/06/2022</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1–2–4–7–15–18</t>
+          <t>2–8–9–13–15–21</t>
         </is>
       </c>
     </row>
@@ -476,12 +476,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>05/24/2022</t>
+          <t>06/03/2022</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2–4–9–13–16–22</t>
+          <t>2–3–4–15–17–24</t>
         </is>
       </c>
     </row>
@@ -491,12 +491,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>05/23/2022</t>
+          <t>06/02/2022</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5–6–7–11–14–21</t>
+          <t>2–6–9–15–21–25</t>
         </is>
       </c>
     </row>
@@ -506,12 +506,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05/20/2022</t>
+          <t>05/31/2022</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4–9–15–18–23–25</t>
+          <t>1–6–7–8–20–25</t>
         </is>
       </c>
     </row>
@@ -521,12 +521,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05/19/2022</t>
+          <t>05/30/2022</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>4–7–9–10–14–16</t>
+          <t>2–7–9–11–12–20</t>
         </is>
       </c>
     </row>
@@ -536,12 +536,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05/17/2022</t>
+          <t>05/27/2022</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1–6–12–13–16–25</t>
+          <t>3–6–8–13–24–25</t>
         </is>
       </c>
     </row>
@@ -551,12 +551,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05/16/2022</t>
+          <t>05/26/2022</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>5–6–8–20–22–25</t>
+          <t>1–2–4–7–15–18</t>
         </is>
       </c>
     </row>
@@ -566,12 +566,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05/13/2022</t>
+          <t>05/24/2022</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2–9–10–12–13–16</t>
+          <t>2–4–9–13–16–22</t>
         </is>
       </c>
     </row>
@@ -581,12 +581,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05/12/2022</t>
+          <t>05/23/2022</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2–4–13–15–18–25</t>
+          <t>5–6–7–11–14–21</t>
         </is>
       </c>
     </row>
@@ -596,12 +596,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>05/10/2022</t>
+          <t>05/20/2022</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2–6–17–19–21–23</t>
+          <t>4–9–15–18–23–25</t>
         </is>
       </c>
     </row>
@@ -611,12 +611,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>05/09/2022</t>
+          <t>05/19/2022</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3–5–10–13–18–20</t>
+          <t>4–7–9–10–14–16</t>
         </is>
       </c>
     </row>
@@ -626,12 +626,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>05/06/2022</t>
+          <t>05/17/2022</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3–7–13–14–24–25</t>
+          <t>1–6–12–13–16–25</t>
         </is>
       </c>
     </row>
@@ -641,12 +641,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>05/05/2022</t>
+          <t>05/16/2022</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3–5–8–17–18–25</t>
+          <t>5–6–8–20–22–25</t>
         </is>
       </c>
     </row>
@@ -656,12 +656,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>05/03/2022</t>
+          <t>05/13/2022</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1–4–13–20–22–25</t>
+          <t>2–9–10–12–13–16</t>
         </is>
       </c>
     </row>
@@ -671,12 +671,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>05/02/2022</t>
+          <t>05/12/2022</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>3–8–17–20–22–25</t>
+          <t>2–4–13–15–18–25</t>
         </is>
       </c>
     </row>
@@ -686,12 +686,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>04/29/2022</t>
+          <t>05/10/2022</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>5–6–12–17–18–23</t>
+          <t>2–6–17–19–21–23</t>
         </is>
       </c>
     </row>
@@ -701,12 +701,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>04/28/2022</t>
+          <t>05/09/2022</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1–5–10–19–20–23</t>
+          <t>3–5–10–13–18–20</t>
         </is>
       </c>
     </row>
@@ -716,12 +716,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>04/26/2022</t>
+          <t>05/06/2022</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1–4–9–15–19–22</t>
+          <t>3–7–13–14–24–25</t>
         </is>
       </c>
     </row>
@@ -731,12 +731,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>04/25/2022</t>
+          <t>05/05/2022</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1–2–9–18–23–24</t>
+          <t>3–5–8–17–18–25</t>
         </is>
       </c>
     </row>
@@ -746,12 +746,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>04/22/2022</t>
+          <t>05/03/2022</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1–8–16–17–19–22</t>
+          <t>1–4–13–20–22–25</t>
         </is>
       </c>
     </row>
@@ -761,12 +761,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>04/21/2022</t>
+          <t>05/02/2022</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>3–11–19–22–23–24</t>
+          <t>3–8–17–20–22–25</t>
         </is>
       </c>
     </row>
@@ -776,12 +776,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>04/19/2022</t>
+          <t>04/29/2022</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>7–8–9–10–16–23</t>
+          <t>5–6–12–17–18–23</t>
         </is>
       </c>
     </row>
@@ -791,12 +791,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>04/18/2022</t>
+          <t>04/28/2022</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1–18–20–21–22–23</t>
+          <t>1–5–10–19–20–23</t>
         </is>
       </c>
     </row>
@@ -806,12 +806,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>04/15/2022</t>
+          <t>04/26/2022</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2–11–14–17–22–23</t>
+          <t>1–4–9–15–19–22</t>
         </is>
       </c>
     </row>
@@ -821,12 +821,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>04/14/2022</t>
+          <t>04/25/2022</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2–3–5–11–21–23</t>
+          <t>1–2–9–18–23–24</t>
         </is>
       </c>
     </row>
@@ -836,12 +836,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>04/12/2022</t>
+          <t>04/22/2022</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>1–6–14–17–19–23</t>
+          <t>1–8–16–17–19–22</t>
         </is>
       </c>
     </row>
@@ -851,12 +851,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>04/11/2022</t>
+          <t>04/21/2022</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>12–13–14–19–21–22</t>
+          <t>3–11–19–22–23–24</t>
         </is>
       </c>
     </row>
@@ -866,12 +866,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>04/08/2022</t>
+          <t>04/19/2022</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>1–2–6–13–15–21</t>
+          <t>7–8–9–10–16–23</t>
         </is>
       </c>
     </row>
@@ -881,12 +881,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>04/07/2022</t>
+          <t>04/18/2022</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>5–10–11–12–14–15</t>
+          <t>1–18–20–21–22–23</t>
         </is>
       </c>
     </row>
@@ -896,12 +896,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>04/05/2022</t>
+          <t>04/15/2022</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2–4–6–13–14–23</t>
+          <t>2–11–14–17–22–23</t>
         </is>
       </c>
     </row>
@@ -911,12 +911,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>04/04/2022</t>
+          <t>04/14/2022</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>5–11–14–15–16–17</t>
+          <t>2–3–5–11–21–23</t>
         </is>
       </c>
     </row>
@@ -926,12 +926,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>04/01/2022</t>
+          <t>04/12/2022</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2–9–16–19–20–21</t>
+          <t>1–6–14–17–19–23</t>
         </is>
       </c>
     </row>
@@ -941,12 +941,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>03/31/2022</t>
+          <t>04/11/2022</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>5–11–13–14–18–22</t>
+          <t>12–13–14–19–21–22</t>
         </is>
       </c>
     </row>
@@ -956,12 +956,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>03/29/2022</t>
+          <t>04/08/2022</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2–4–9–16–18–19</t>
+          <t>1–2–6–13–15–21</t>
         </is>
       </c>
     </row>
@@ -971,12 +971,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>03/28/2022</t>
+          <t>04/07/2022</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>5–9–10–15–21–22</t>
+          <t>5–10–11–12–14–15</t>
         </is>
       </c>
     </row>
@@ -986,12 +986,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>03/25/2022</t>
+          <t>04/05/2022</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>6–7–16–18–23–25</t>
+          <t>2–4–6–13–14–23</t>
         </is>
       </c>
     </row>
@@ -1001,12 +1001,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>03/24/2022</t>
+          <t>04/04/2022</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>5–9–15–16–17–21</t>
+          <t>5–11–14–15–16–17</t>
         </is>
       </c>
     </row>
@@ -1016,12 +1016,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>03/22/2022</t>
+          <t>04/01/2022</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2–6–10–11–16–23</t>
+          <t>2–9–16–19–20–21</t>
         </is>
       </c>
     </row>
@@ -1031,12 +1031,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>03/21/2022</t>
+          <t>03/31/2022</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>6–9–14–16–22–23</t>
+          <t>5–11–13–14–18–22</t>
         </is>
       </c>
     </row>
@@ -1046,12 +1046,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>03/18/2022</t>
+          <t>03/29/2022</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>1–4–19–20–23–25</t>
+          <t>2–4–9–16–18–19</t>
         </is>
       </c>
     </row>
@@ -1061,12 +1061,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>03/17/2022</t>
+          <t>03/28/2022</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>1–3–4–5–8–16</t>
+          <t>5–9–10–15–21–22</t>
         </is>
       </c>
     </row>
@@ -1076,12 +1076,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>03/15/2022</t>
+          <t>03/25/2022</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>5–9–16–17–19–21</t>
+          <t>6–7–16–18–23–25</t>
         </is>
       </c>
     </row>
@@ -1091,12 +1091,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>03/14/2022</t>
+          <t>03/24/2022</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>1–4–7–13–16–24</t>
+          <t>5–9–15–16–17–21</t>
         </is>
       </c>
     </row>
@@ -1106,12 +1106,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>03/11/2022</t>
+          <t>03/22/2022</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>6–13–15–18–21–23</t>
+          <t>2–6–10–11–16–23</t>
         </is>
       </c>
     </row>
@@ -1121,12 +1121,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>03/10/2022</t>
+          <t>03/21/2022</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2–4–15–16–19–21</t>
+          <t>6–9–14–16–22–23</t>
         </is>
       </c>
     </row>
@@ -1136,12 +1136,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>03/08/2022</t>
+          <t>03/18/2022</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>1–3–4–7–10–20</t>
+          <t>1–4–19–20–23–25</t>
         </is>
       </c>
     </row>
@@ -1151,12 +1151,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>03/07/2022</t>
+          <t>03/17/2022</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>1–4–8–15–24–25</t>
+          <t>1–3–4–5–8–16</t>
         </is>
       </c>
     </row>
@@ -1166,12 +1166,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>03/04/2022</t>
+          <t>03/15/2022</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2–5–9–12–18–24</t>
+          <t>5–9–16–17–19–21</t>
         </is>
       </c>
     </row>
@@ -1181,12 +1181,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>03/03/2022</t>
+          <t>03/14/2022</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>6–7–9–12–14–22</t>
+          <t>1–4–7–13–16–24</t>
         </is>
       </c>
     </row>
@@ -1196,12 +1196,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>03/01/2022</t>
+          <t>03/11/2022</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2–7–9–14–16–20</t>
+          <t>6–13–15–18–21–23</t>
         </is>
       </c>
     </row>
@@ -1211,12 +1211,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>02/28/2022</t>
+          <t>03/10/2022</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>1–6–7–19–22–24</t>
+          <t>2–4–15–16–19–21</t>
         </is>
       </c>
     </row>
@@ -1226,12 +1226,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>02/25/2022</t>
+          <t>03/08/2022</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>3–7–9–14–15–22</t>
+          <t>1–3–4–7–10–20</t>
         </is>
       </c>
     </row>
@@ -1241,12 +1241,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>02/24/2022</t>
+          <t>03/07/2022</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>5–13–14–15–22–24</t>
+          <t>1–4–8–15–24–25</t>
         </is>
       </c>
     </row>
@@ -1256,12 +1256,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>02/22/2022</t>
+          <t>03/04/2022</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>6–9–18–20–22–23</t>
+          <t>2–5–9–12–18–24</t>
         </is>
       </c>
     </row>
@@ -1271,12 +1271,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>02/21/2022</t>
+          <t>03/03/2022</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>3–11–15–16–17–21</t>
+          <t>6–7–9–12–14–22</t>
         </is>
       </c>
     </row>
@@ -1286,12 +1286,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>02/18/2022</t>
+          <t>03/01/2022</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>1–2–10–14–22–23</t>
+          <t>2–7–9–14–16–20</t>
         </is>
       </c>
     </row>
@@ -1301,12 +1301,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>02/17/2022</t>
+          <t>02/28/2022</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>3–4–10–19–22–24</t>
+          <t>1–6–7–19–22–24</t>
         </is>
       </c>
     </row>
@@ -1316,12 +1316,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>02/15/2022</t>
+          <t>02/25/2022</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>1–9–13–15–19–20</t>
+          <t>3–7–9–14–15–22</t>
         </is>
       </c>
     </row>
@@ -1331,12 +1331,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>02/14/2022</t>
+          <t>02/24/2022</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>4–7–9–10–14–17</t>
+          <t>5–13–14–15–22–24</t>
         </is>
       </c>
     </row>
@@ -1346,12 +1346,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>02/11/2022</t>
+          <t>02/22/2022</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>4–6–8–10–12–20</t>
+          <t>6–9–18–20–22–23</t>
         </is>
       </c>
     </row>
@@ -1361,12 +1361,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>02/10/2022</t>
+          <t>02/21/2022</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>5–11–16–20–22–23</t>
+          <t>3–11–15–16–17–21</t>
         </is>
       </c>
     </row>
@@ -1376,12 +1376,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>02/08/2022</t>
+          <t>02/18/2022</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2–5–14–16–17–25</t>
+          <t>1–2–10–14–22–23</t>
         </is>
       </c>
     </row>
@@ -1391,12 +1391,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>02/07/2022</t>
+          <t>02/17/2022</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>4–7–14–16–18–23</t>
+          <t>3–4–10–19–22–24</t>
         </is>
       </c>
     </row>
@@ -1406,12 +1406,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>02/04/2022</t>
+          <t>02/15/2022</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>13–17–20–23–24–25</t>
+          <t>1–9–13–15–19–20</t>
         </is>
       </c>
     </row>
@@ -1421,12 +1421,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>02/03/2022</t>
+          <t>02/14/2022</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>6–12–14–17–22–25</t>
+          <t>4–7–9–10–14–17</t>
         </is>
       </c>
     </row>
@@ -1436,12 +1436,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>02/01/2022</t>
+          <t>02/11/2022</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>6–7–12–15–16–20</t>
+          <t>4–6–8–10–12–20</t>
         </is>
       </c>
     </row>
@@ -1451,12 +1451,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>01/31/2022</t>
+          <t>02/10/2022</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>5–7–8–9–10–22</t>
+          <t>5–11–16–20–22–23</t>
         </is>
       </c>
     </row>
@@ -1466,12 +1466,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>01/28/2022</t>
+          <t>02/08/2022</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>7–9–11–12–17–19</t>
+          <t>2–5–14–16–17–25</t>
         </is>
       </c>
     </row>
@@ -1481,12 +1481,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>01/27/2022</t>
+          <t>02/07/2022</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2–3–14–19–20–21</t>
+          <t>4–7–14–16–18–23</t>
         </is>
       </c>
     </row>
@@ -1496,12 +1496,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>01/25/2022</t>
+          <t>02/04/2022</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>3–4–5–11–17–19</t>
+          <t>13–17–20–23–24–25</t>
         </is>
       </c>
     </row>
@@ -1511,12 +1511,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>01/24/2022</t>
+          <t>02/03/2022</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>4–7–8–20–21–25</t>
+          <t>6–12–14–17–22–25</t>
         </is>
       </c>
     </row>
@@ -1526,12 +1526,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>01/21/2022</t>
+          <t>02/01/2022</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>8–11–14–15–18–24</t>
+          <t>6–7–12–15–16–20</t>
         </is>
       </c>
     </row>
@@ -1541,12 +1541,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>01/20/2022</t>
+          <t>01/31/2022</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2–15–19–20–22–24</t>
+          <t>5–7–8–9–10–22</t>
         </is>
       </c>
     </row>
@@ -1556,12 +1556,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>01/18/2022</t>
+          <t>01/28/2022</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>3–5–16–17–18–21</t>
+          <t>7–9–11–12–17–19</t>
         </is>
       </c>
     </row>
@@ -1571,12 +1571,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>01/17/2022</t>
+          <t>01/27/2022</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>5–8–16–18–20–22</t>
+          <t>2–3–14–19–20–21</t>
         </is>
       </c>
     </row>
@@ -1586,12 +1586,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>01/14/2022</t>
+          <t>01/25/2022</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2–5–8–9–10–13</t>
+          <t>3–4–5–11–17–19</t>
         </is>
       </c>
     </row>
@@ -1601,12 +1601,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>01/13/2022</t>
+          <t>01/24/2022</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2–6–8–11–18–21</t>
+          <t>4–7–8–20–21–25</t>
         </is>
       </c>
     </row>
@@ -1616,12 +1616,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>01/11/2022</t>
+          <t>01/21/2022</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>7–8–9–15–19–23</t>
+          <t>8–11–14–15–18–24</t>
         </is>
       </c>
     </row>
@@ -1631,12 +1631,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>01/10/2022</t>
+          <t>01/20/2022</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>10–13–14–19–22–23</t>
+          <t>2–15–19–20–22–24</t>
         </is>
       </c>
     </row>
@@ -1646,12 +1646,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>01/07/2022</t>
+          <t>01/18/2022</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>4–8–21–23–24–25</t>
+          <t>3–5–16–17–18–21</t>
         </is>
       </c>
     </row>
@@ -1661,12 +1661,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>01/06/2022</t>
+          <t>01/17/2022</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>7–9–10–17–18–23</t>
+          <t>5–8–16–18–20–22</t>
         </is>
       </c>
     </row>
@@ -1676,12 +1676,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>01/04/2022</t>
+          <t>01/14/2022</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>4–7–14–15–24–25</t>
+          <t>2–5–8–9–10–13</t>
         </is>
       </c>
     </row>
@@ -1691,12 +1691,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>01/03/2022</t>
+          <t>01/13/2022</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>6–10–17–18–19–21</t>
+          <t>2–6–8–11–18–21</t>
         </is>
       </c>
     </row>
@@ -1706,12 +1706,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>12/31/2021</t>
+          <t>01/11/2022</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>11–17–20–22–23–24</t>
+          <t>7–8–9–15–19–23</t>
         </is>
       </c>
     </row>
@@ -1721,12 +1721,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>12/30/2021</t>
+          <t>01/10/2022</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>1–8–9–13–20–25</t>
+          <t>10–13–14–19–22–23</t>
         </is>
       </c>
     </row>
@@ -1736,12 +1736,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>12/28/2021</t>
+          <t>01/07/2022</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>4–9–11–15–16–25</t>
+          <t>4–8–21–23–24–25</t>
         </is>
       </c>
     </row>
@@ -1751,12 +1751,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>12/27/2021</t>
+          <t>01/06/2022</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>3–4–10–14–19–25</t>
+          <t>7–9–10–17–18–23</t>
         </is>
       </c>
     </row>
@@ -1766,12 +1766,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>12/24/2021</t>
+          <t>01/04/2022</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>4–6–13–17–21–22</t>
+          <t>4–7–14–15–24–25</t>
         </is>
       </c>
     </row>
@@ -1781,12 +1781,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>12/23/2021</t>
+          <t>01/03/2022</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>1–2–3–15–20–23</t>
+          <t>6–10–17–18–19–21</t>
         </is>
       </c>
     </row>
@@ -1796,12 +1796,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>12/21/2021</t>
+          <t>12/31/2021</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>6–9–11–12–14–25</t>
+          <t>11–17–20–22–23–24</t>
         </is>
       </c>
     </row>
@@ -1811,12 +1811,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>12/20/2021</t>
+          <t>12/30/2021</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>7–8–9–22–23–24</t>
+          <t>1–8–9–13–20–25</t>
         </is>
       </c>
     </row>
@@ -1826,12 +1826,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>12/17/2021</t>
+          <t>12/28/2021</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>3–9–15–16–18–22</t>
+          <t>4–9–11–15–16–25</t>
         </is>
       </c>
     </row>
@@ -1841,12 +1841,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>12/16/2021</t>
+          <t>12/27/2021</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2–3–11–13–24–25</t>
+          <t>3–4–10–14–19–25</t>
         </is>
       </c>
     </row>
@@ -1856,12 +1856,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>12/14/2021</t>
+          <t>12/24/2021</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2–7–9–17–23–24</t>
+          <t>4–6–13–17–21–22</t>
         </is>
       </c>
     </row>
@@ -1871,12 +1871,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>12/13/2021</t>
+          <t>12/23/2021</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2–6–15–16–23–24</t>
+          <t>1–2–3–15–20–23</t>
         </is>
       </c>
     </row>
@@ -1886,12 +1886,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>12/10/2021</t>
+          <t>12/21/2021</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>3–6–9–10–14–21</t>
+          <t>6–9–11–12–14–25</t>
         </is>
       </c>
     </row>
@@ -1901,12 +1901,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>12/09/2021</t>
+          <t>12/20/2021</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2–12–14–15–19–21</t>
+          <t>7–8–9–22–23–24</t>
         </is>
       </c>
     </row>
@@ -1916,12 +1916,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>12/07/2021</t>
+          <t>12/17/2021</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>3–5–8–9–16–25</t>
+          <t>3–9–15–16–18–22</t>
         </is>
       </c>
     </row>
@@ -1931,12 +1931,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>12/06/2021</t>
+          <t>12/16/2021</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>3–5–8–12–15–19</t>
+          <t>2–3–11–13–24–25</t>
         </is>
       </c>
     </row>
@@ -1946,12 +1946,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>12/03/2021</t>
+          <t>12/14/2021</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10–13–14–15–21–24</t>
+          <t>2–7–9–17–23–24</t>
         </is>
       </c>
     </row>
@@ -1961,12 +1961,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>12/02/2021</t>
+          <t>12/13/2021</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2–7–8–11–22–24</t>
+          <t>2–6–15–16–23–24</t>
         </is>
       </c>
     </row>
@@ -1976,12 +1976,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>11/30/2021</t>
+          <t>12/10/2021</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>12–14–20–23–24–25</t>
+          <t>3–6–9–10–14–21</t>
         </is>
       </c>
     </row>
@@ -1991,12 +1991,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>11/29/2021</t>
+          <t>12/09/2021</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>4–8–10–13–20–21</t>
+          <t>2–12–14–15–19–21</t>
         </is>
       </c>
     </row>
@@ -2006,12 +2006,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>11/26/2021</t>
+          <t>12/07/2021</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>3–7–14–17–24–25</t>
+          <t>3–5–8–9–16–25</t>
         </is>
       </c>
     </row>
@@ -2021,12 +2021,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>11/25/2021</t>
+          <t>12/06/2021</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2–11–16–18–20–21</t>
+          <t>3–5–8–12–15–19</t>
         </is>
       </c>
     </row>
@@ -2036,12 +2036,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>11/23/2021</t>
+          <t>12/03/2021</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2–10–11–12–14–19</t>
+          <t>10–13–14–15–21–24</t>
         </is>
       </c>
     </row>
@@ -2051,12 +2051,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>11/22/2021</t>
+          <t>12/02/2021</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>5–10–12–16–20–25</t>
+          <t>2–7–8–11–22–24</t>
         </is>
       </c>
     </row>
@@ -2066,12 +2066,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>11/19/2021</t>
+          <t>11/30/2021</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>12–16–19–20–21–24</t>
+          <t>12–14–20–23–24–25</t>
         </is>
       </c>
     </row>
@@ -2081,12 +2081,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>11/18/2021</t>
+          <t>11/29/2021</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>1–4–17–18–20–23</t>
+          <t>4–8–10–13–20–21</t>
         </is>
       </c>
     </row>
@@ -2096,12 +2096,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>11/16/2021</t>
+          <t>11/26/2021</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>5–8–10–11–16–23</t>
+          <t>3–7–14–17–24–25</t>
         </is>
       </c>
     </row>
@@ -2111,12 +2111,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>11/15/2021</t>
+          <t>11/25/2021</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2–6–10–11–15–18</t>
+          <t>2–11–16–18–20–21</t>
         </is>
       </c>
     </row>
@@ -2126,12 +2126,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>11/12/2021</t>
+          <t>11/23/2021</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>1–13–14–15–22–25</t>
+          <t>2–10–11–12–14–19</t>
         </is>
       </c>
     </row>
@@ -2141,12 +2141,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>11/11/2021</t>
+          <t>11/22/2021</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2–3–5–14–21–22</t>
+          <t>5–10–12–16–20–25</t>
         </is>
       </c>
     </row>
@@ -2156,12 +2156,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>11/09/2021</t>
+          <t>11/19/2021</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2–4–10–13–16–23</t>
+          <t>12–16–19–20–21–24</t>
         </is>
       </c>
     </row>
@@ -2171,12 +2171,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>11/08/2021</t>
+          <t>11/18/2021</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>1–2–8–10–13–24</t>
+          <t>1–4–17–18–20–23</t>
         </is>
       </c>
     </row>
@@ -2186,12 +2186,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>11/05/2021</t>
+          <t>11/16/2021</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>4–11–12–18–19–25</t>
+          <t>5–8–10–11–16–23</t>
         </is>
       </c>
     </row>
@@ -2201,12 +2201,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>11/04/2021</t>
+          <t>11/15/2021</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>10–15–19–21–24–25</t>
+          <t>2–6–10–11–15–18</t>
         </is>
       </c>
     </row>
@@ -2216,12 +2216,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>11/02/2021</t>
+          <t>11/12/2021</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>3–4–9–16–17–18</t>
+          <t>1–13–14–15–22–25</t>
         </is>
       </c>
     </row>
@@ -2231,12 +2231,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>11/01/2021</t>
+          <t>11/11/2021</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>5–6–14–15–18–20</t>
+          <t>2–3–5–14–21–22</t>
         </is>
       </c>
     </row>
@@ -2246,12 +2246,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>10/29/2021</t>
+          <t>11/09/2021</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2–3–8–9–13–15</t>
+          <t>2–4–10–13–16–23</t>
         </is>
       </c>
     </row>
@@ -2261,12 +2261,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>10/28/2021</t>
+          <t>11/08/2021</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>7–15–19–20–23–24</t>
+          <t>1–2–8–10–13–24</t>
         </is>
       </c>
     </row>
@@ -2276,12 +2276,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>10/26/2021</t>
+          <t>11/05/2021</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>3–4–14–16–17–25</t>
+          <t>4–11–12–18–19–25</t>
         </is>
       </c>
     </row>
@@ -2291,12 +2291,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>10/25/2021</t>
+          <t>11/04/2021</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>9–12–17–19–20–24</t>
+          <t>10–15–19–21–24–25</t>
         </is>
       </c>
     </row>
@@ -2306,12 +2306,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>10/22/2021</t>
+          <t>11/02/2021</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2–5–6–18–20–23</t>
+          <t>3–4–9–16–17–18</t>
         </is>
       </c>
     </row>
@@ -2321,12 +2321,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>10/21/2021</t>
+          <t>11/01/2021</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>5–8–9–13–22–24</t>
+          <t>5–6–14–15–18–20</t>
         </is>
       </c>
     </row>
@@ -2336,12 +2336,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>10/19/2021</t>
+          <t>10/29/2021</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>8–9–11–15–19–25</t>
+          <t>2–3–8–9–13–15</t>
         </is>
       </c>
     </row>
@@ -2351,12 +2351,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>10/18/2021</t>
+          <t>10/28/2021</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>3–4–8–10–12–20</t>
+          <t>7–15–19–20–23–24</t>
         </is>
       </c>
     </row>
@@ -2366,12 +2366,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>10/15/2021</t>
+          <t>10/26/2021</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>1–3–4–8–19–21</t>
+          <t>3–4–14–16–17–25</t>
         </is>
       </c>
     </row>
@@ -2381,12 +2381,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>10/14/2021</t>
+          <t>10/25/2021</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2–5–8–15–16–23</t>
+          <t>9–12–17–19–20–24</t>
         </is>
       </c>
     </row>
@@ -2396,12 +2396,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>10/12/2021</t>
+          <t>10/22/2021</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>5–6–13–14–24–25</t>
+          <t>2–5–6–18–20–23</t>
         </is>
       </c>
     </row>
@@ -2411,12 +2411,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>10/11/2021</t>
+          <t>10/21/2021</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>1–2–3–5–21–23</t>
+          <t>5–8–9–13–22–24</t>
         </is>
       </c>
     </row>
@@ -2426,12 +2426,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>10/08/2021</t>
+          <t>10/19/2021</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>10–11–13–17–20–22</t>
+          <t>8–9–11–15–19–25</t>
         </is>
       </c>
     </row>
@@ -2441,12 +2441,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>10/07/2021</t>
+          <t>10/18/2021</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>3–5–8–16–19–23</t>
+          <t>3–4–8–10–12–20</t>
         </is>
       </c>
     </row>
@@ -2456,12 +2456,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>10/05/2021</t>
+          <t>10/15/2021</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>7–9–13–15–18–23</t>
+          <t>1–3–4–8–19–21</t>
         </is>
       </c>
     </row>
@@ -2471,12 +2471,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>10/04/2021</t>
+          <t>10/14/2021</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>8–9–11–18–20–23</t>
+          <t>2–5–8–15–16–23</t>
         </is>
       </c>
     </row>
@@ -2486,12 +2486,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>10/01/2021</t>
+          <t>10/12/2021</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2–3–5–7–11–18</t>
+          <t>5–6–13–14–24–25</t>
         </is>
       </c>
     </row>
@@ -2501,12 +2501,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>09/30/2021</t>
+          <t>10/11/2021</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>5–16–18–20–22–24</t>
+          <t>1–2–3–5–21–23</t>
         </is>
       </c>
     </row>
@@ -2516,12 +2516,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>09/28/2021</t>
+          <t>10/08/2021</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>1–9–11–12–18–22</t>
+          <t>10–11–13–17–20–22</t>
         </is>
       </c>
     </row>
@@ -2531,12 +2531,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>09/27/2021</t>
+          <t>10/07/2021</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>4–5–6–10–14–22</t>
+          <t>3–5–8–16–19–23</t>
         </is>
       </c>
     </row>
@@ -2546,12 +2546,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>09/24/2021</t>
+          <t>10/05/2021</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>4–11–15–16–22–25</t>
+          <t>7–9–13–15–18–23</t>
         </is>
       </c>
     </row>
@@ -2561,12 +2561,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>09/23/2021</t>
+          <t>10/04/2021</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>4–9–13–15–17–18</t>
+          <t>8–9–11–18–20–23</t>
         </is>
       </c>
     </row>
@@ -2576,12 +2576,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>09/21/2021</t>
+          <t>10/01/2021</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>1–13–14–21–22–24</t>
+          <t>2–3–5–7–11–18</t>
         </is>
       </c>
     </row>
@@ -2591,12 +2591,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>09/20/2021</t>
+          <t>09/30/2021</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>1–13–17–18–20–22</t>
+          <t>5–16–18–20–22–24</t>
         </is>
       </c>
     </row>
@@ -2606,12 +2606,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>09/17/2021</t>
+          <t>09/28/2021</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2–6–8–9–11–12</t>
+          <t>1–9–11–12–18–22</t>
         </is>
       </c>
     </row>
@@ -2621,12 +2621,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>09/16/2021</t>
+          <t>09/27/2021</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2–11–12–14–17–19</t>
+          <t>4–5–6–10–14–22</t>
         </is>
       </c>
     </row>
@@ -2636,12 +2636,12 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>09/14/2021</t>
+          <t>09/24/2021</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>4–11–18–19–20–23</t>
+          <t>4–11–15–16–22–25</t>
         </is>
       </c>
     </row>
@@ -2651,12 +2651,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>09/13/2021</t>
+          <t>09/23/2021</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>1–8–11–12–13–18</t>
+          <t>4–9–13–15–17–18</t>
         </is>
       </c>
     </row>
@@ -2666,12 +2666,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>09/10/2021</t>
+          <t>09/21/2021</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>3–4–6–8–11–16</t>
+          <t>1–13–14–21–22–24</t>
         </is>
       </c>
     </row>
@@ -2681,12 +2681,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>09/09/2021</t>
+          <t>09/20/2021</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>1–14–15–20–21–25</t>
+          <t>1–13–17–18–20–22</t>
         </is>
       </c>
     </row>
@@ -2696,12 +2696,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>09/07/2021</t>
+          <t>09/17/2021</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>5–7–8–9–18–21</t>
+          <t>2–6–8–9–11–12</t>
         </is>
       </c>
     </row>
@@ -2711,12 +2711,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>09/06/2021</t>
+          <t>09/16/2021</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>6–7–9–16–21–22</t>
+          <t>2–11–12–14–17–19</t>
         </is>
       </c>
     </row>
@@ -2726,12 +2726,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>09/03/2021</t>
+          <t>09/14/2021</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>1–3–11–21–22–24</t>
+          <t>4–11–18–19–20–23</t>
         </is>
       </c>
     </row>
@@ -2741,12 +2741,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>09/02/2021</t>
+          <t>09/13/2021</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>1–2–4–10–11–24</t>
+          <t>1–8–11–12–13–18</t>
         </is>
       </c>
     </row>
@@ -2756,12 +2756,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>08/31/2021</t>
+          <t>09/10/2021</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>1–8–9–15–19–21</t>
+          <t>3–4–6–8–11–16</t>
         </is>
       </c>
     </row>
@@ -2771,12 +2771,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>08/30/2021</t>
+          <t>09/09/2021</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>5–10–19–20–21–25</t>
+          <t>1–14–15–20–21–25</t>
         </is>
       </c>
     </row>
@@ -2786,12 +2786,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>08/27/2021</t>
+          <t>09/07/2021</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>1–10–15–17–18–21</t>
+          <t>5–7–8–9–18–21</t>
         </is>
       </c>
     </row>
@@ -2801,12 +2801,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>08/26/2021</t>
+          <t>09/06/2021</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>6–14–18–19–23–25</t>
+          <t>6–7–9–16–21–22</t>
         </is>
       </c>
     </row>
@@ -2816,12 +2816,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>08/24/2021</t>
+          <t>09/03/2021</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2–3–6–20–21–23</t>
+          <t>1–3–11–21–22–24</t>
         </is>
       </c>
     </row>
@@ -2831,12 +2831,12 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>08/23/2021</t>
+          <t>09/02/2021</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>9–11–12–14–18–23</t>
+          <t>1–2–4–10–11–24</t>
         </is>
       </c>
     </row>
@@ -2846,12 +2846,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>08/20/2021</t>
+          <t>08/31/2021</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>5–8–17–19–20–24</t>
+          <t>1–8–9–15–19–21</t>
         </is>
       </c>
     </row>
@@ -2861,12 +2861,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>08/19/2021</t>
+          <t>08/30/2021</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2–3–6–8–12–21</t>
+          <t>5–10–19–20–21–25</t>
         </is>
       </c>
     </row>
@@ -2876,12 +2876,12 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>08/17/2021</t>
+          <t>08/27/2021</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>7–12–15–16–20–25</t>
+          <t>1–10–15–17–18–21</t>
         </is>
       </c>
     </row>
@@ -2891,12 +2891,12 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>08/16/2021</t>
+          <t>08/26/2021</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>1–3–5–8–9–15</t>
+          <t>6–14–18–19–23–25</t>
         </is>
       </c>
     </row>
@@ -2906,12 +2906,12 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>08/13/2021</t>
+          <t>08/24/2021</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>1–5–10–14–18–24</t>
+          <t>2–3–6–20–21–23</t>
         </is>
       </c>
     </row>
@@ -2921,12 +2921,12 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>08/12/2021</t>
+          <t>08/23/2021</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>4–7–13–17–21–22</t>
+          <t>9–11–12–14–18–23</t>
         </is>
       </c>
     </row>
@@ -2936,12 +2936,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>08/10/2021</t>
+          <t>08/20/2021</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>4–6–9–10–15–24</t>
+          <t>5–8–17–19–20–24</t>
         </is>
       </c>
     </row>
@@ -2951,12 +2951,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>08/09/2021</t>
+          <t>08/19/2021</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>1–2–6–13–18–25</t>
+          <t>2–3–6–8–12–21</t>
         </is>
       </c>
     </row>
@@ -2966,12 +2966,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>08/06/2021</t>
+          <t>08/17/2021</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>5–8–9–14–23–24</t>
+          <t>7–12–15–16–20–25</t>
         </is>
       </c>
     </row>
@@ -2981,12 +2981,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>08/05/2021</t>
+          <t>08/16/2021</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2–5–6–12–14–18</t>
+          <t>1–3–5–8–9–15</t>
         </is>
       </c>
     </row>
@@ -2996,12 +2996,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>08/03/2021</t>
+          <t>08/13/2021</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2–7–17–22–24–25</t>
+          <t>1–5–10–14–18–24</t>
         </is>
       </c>
     </row>
@@ -3011,12 +3011,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>08/02/2021</t>
+          <t>08/12/2021</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>7–12–13–18–22–24</t>
+          <t>4–7–13–17–21–22</t>
         </is>
       </c>
     </row>
@@ -3026,12 +3026,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>07/30/2021</t>
+          <t>08/10/2021</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>3–4–13–22–24–25</t>
+          <t>4–6–9–10–15–24</t>
         </is>
       </c>
     </row>
@@ -3041,12 +3041,12 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>07/29/2021</t>
+          <t>08/09/2021</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>5–7–12–17–19–24</t>
+          <t>1–2–6–13–18–25</t>
         </is>
       </c>
     </row>
@@ -3056,12 +3056,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>07/27/2021</t>
+          <t>08/06/2021</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>1–4–16–17–18–21</t>
+          <t>5–8–9–14–23–24</t>
         </is>
       </c>
     </row>
@@ -3071,12 +3071,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>07/26/2021</t>
+          <t>08/05/2021</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>3–14–19–21–23–24</t>
+          <t>2–5–6–12–14–18</t>
         </is>
       </c>
     </row>
@@ -3086,12 +3086,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>07/23/2021</t>
+          <t>08/03/2021</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>9–12–14–16–22–25</t>
+          <t>2–7–17–22–24–25</t>
         </is>
       </c>
     </row>
@@ -3101,12 +3101,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>07/22/2021</t>
+          <t>08/02/2021</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2–5–6–15–16–20</t>
+          <t>7–12–13–18–22–24</t>
         </is>
       </c>
     </row>
@@ -3116,12 +3116,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>07/20/2021</t>
+          <t>07/30/2021</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>4–7–12–15–20–21</t>
+          <t>3–4–13–22–24–25</t>
         </is>
       </c>
     </row>
@@ -3131,12 +3131,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>07/19/2021</t>
+          <t>07/29/2021</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2–5–9–10–18–22</t>
+          <t>5–7–12–17–19–24</t>
         </is>
       </c>
     </row>
@@ -3146,12 +3146,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>07/16/2021</t>
+          <t>07/27/2021</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>4–8–10–11–12–21</t>
+          <t>1–4–16–17–18–21</t>
         </is>
       </c>
     </row>
@@ -3161,12 +3161,12 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>07/15/2021</t>
+          <t>07/26/2021</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>1–6–9–11–17–22</t>
+          <t>3–14–19–21–23–24</t>
         </is>
       </c>
     </row>
@@ -3176,12 +3176,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>07/13/2021</t>
+          <t>07/23/2021</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>4–11–14–15–17–18</t>
+          <t>9–12–14–16–22–25</t>
         </is>
       </c>
     </row>
@@ -3191,12 +3191,12 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>07/12/2021</t>
+          <t>07/22/2021</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>1–4–5–7–8–22</t>
+          <t>2–5–6–15–16–20</t>
         </is>
       </c>
     </row>
@@ -3206,12 +3206,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>07/09/2021</t>
+          <t>07/20/2021</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>7–13–14–16–21–22</t>
+          <t>4–7–12–15–20–21</t>
         </is>
       </c>
     </row>
@@ -3221,12 +3221,12 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>07/08/2021</t>
+          <t>07/19/2021</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>5–8–9–13–14–16</t>
+          <t>2–5–9–10–18–22</t>
         </is>
       </c>
     </row>
@@ -3236,12 +3236,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>07/06/2021</t>
+          <t>07/16/2021</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>1–18–20–21–22–25</t>
+          <t>4–8–10–11–12–21</t>
         </is>
       </c>
     </row>
@@ -3251,12 +3251,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>07/05/2021</t>
+          <t>07/15/2021</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>3–7–11–12–13–23</t>
+          <t>1–6–9–11–17–22</t>
         </is>
       </c>
     </row>
@@ -3266,12 +3266,12 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>07/02/2021</t>
+          <t>07/13/2021</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>1–4–5–8–14–20</t>
+          <t>4–11–14–15–17–18</t>
         </is>
       </c>
     </row>
@@ -3281,12 +3281,12 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>07/01/2021</t>
+          <t>07/12/2021</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>6–9–11–14–16–19</t>
+          <t>1–4–5–7–8–22</t>
         </is>
       </c>
     </row>
@@ -3296,12 +3296,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>06/29/2021</t>
+          <t>07/09/2021</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>1–5–9–10–16–20</t>
+          <t>7–13–14–16–21–22</t>
         </is>
       </c>
     </row>
@@ -3311,12 +3311,12 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>06/28/2021</t>
+          <t>07/08/2021</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>4–14–18–20–21–22</t>
+          <t>5–8–9–13–14–16</t>
         </is>
       </c>
     </row>
@@ -3326,12 +3326,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>06/25/2021</t>
+          <t>07/06/2021</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>1–3–4–7–11–18</t>
+          <t>1–18–20–21–22–25</t>
         </is>
       </c>
     </row>
@@ -3341,12 +3341,12 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>06/24/2021</t>
+          <t>07/05/2021</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>1–5–9–11–20–22</t>
+          <t>3–7–11–12–13–23</t>
         </is>
       </c>
     </row>
@@ -3356,12 +3356,12 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>06/22/2021</t>
+          <t>07/02/2021</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>7–9–12–18–21–23</t>
+          <t>1–4–5–8–14–20</t>
         </is>
       </c>
     </row>
@@ -3371,12 +3371,12 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>06/21/2021</t>
+          <t>07/01/2021</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>7–11–17–18–23–24</t>
+          <t>6–9–11–14–16–19</t>
         </is>
       </c>
     </row>
@@ -3386,12 +3386,12 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>06/18/2021</t>
+          <t>06/29/2021</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2–7–11–17–18–25</t>
+          <t>1–5–9–10–16–20</t>
         </is>
       </c>
     </row>
@@ -3401,12 +3401,12 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>06/17/2021</t>
+          <t>06/28/2021</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>3–12–17–19–24–25</t>
+          <t>4–14–18–20–21–22</t>
         </is>
       </c>
     </row>
@@ -3416,12 +3416,12 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>06/15/2021</t>
+          <t>06/25/2021</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>3–5–12–16–18–23</t>
+          <t>1–3–4–7–11–18</t>
         </is>
       </c>
     </row>
@@ -3431,12 +3431,12 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>06/14/2021</t>
+          <t>06/24/2021</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>1–5–11–12–22–23</t>
+          <t>1–5–9–11–20–22</t>
         </is>
       </c>
     </row>
@@ -3446,12 +3446,12 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>06/11/2021</t>
+          <t>06/22/2021</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2–5–10–11–24–25</t>
+          <t>7–9–12–18–21–23</t>
         </is>
       </c>
     </row>
@@ -3461,12 +3461,12 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>06/10/2021</t>
+          <t>06/21/2021</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>7–10–13–14–18–21</t>
+          <t>7–11–17–18–23–24</t>
         </is>
       </c>
     </row>
@@ -3476,12 +3476,12 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>06/08/2021</t>
+          <t>06/18/2021</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>8–9–15–16–23–25</t>
+          <t>2–7–11–17–18–25</t>
         </is>
       </c>
     </row>
@@ -3491,12 +3491,12 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>06/07/2021</t>
+          <t>06/17/2021</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>4–6–7–11–17–20</t>
+          <t>3–12–17–19–24–25</t>
         </is>
       </c>
     </row>
@@ -3506,12 +3506,12 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>06/04/2021</t>
+          <t>06/15/2021</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>1–2–9–15–18–24</t>
+          <t>3–5–12–16–18–23</t>
         </is>
       </c>
     </row>
@@ -3521,12 +3521,12 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>06/03/2021</t>
+          <t>06/14/2021</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>5–6–8–15–19–22</t>
+          <t>1–5–11–12–22–23</t>
         </is>
       </c>
     </row>
@@ -3536,12 +3536,12 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>06/01/2021</t>
+          <t>06/11/2021</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>4–7–12–14–21–22</t>
+          <t>2–5–10–11–24–25</t>
         </is>
       </c>
     </row>
@@ -3551,12 +3551,12 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>05/31/2021</t>
+          <t>06/10/2021</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>3–4–17–18–22–23</t>
+          <t>7–10–13–14–18–21</t>
         </is>
       </c>
     </row>
@@ -3566,12 +3566,12 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>05/28/2021</t>
+          <t>06/08/2021</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>1–3–7–11–12–14</t>
+          <t>8–9–15–16–23–25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
final touches, paypal button, spelling errors, donate & twitter links, etc
</commit_message>
<xml_diff>
--- a/lottopy_site/lottopy/lottopy_web_edition/cash25.xlsx
+++ b/lottopy_site/lottopy/lottopy_web_edition/cash25.xlsx
@@ -446,12 +446,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>06/07/2022</t>
+          <t>06/10/2022</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2–8–10–11–12–22</t>
+          <t>1–3–4–13–14–22</t>
         </is>
       </c>
     </row>
@@ -461,12 +461,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>06/06/2022</t>
+          <t>06/09/2022</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2–8–9–13–15–21</t>
+          <t>8–10–11–12–22–25</t>
         </is>
       </c>
     </row>
@@ -476,12 +476,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>06/03/2022</t>
+          <t>06/07/2022</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2–3–4–15–17–24</t>
+          <t>2–8–10–11–12–22</t>
         </is>
       </c>
     </row>
@@ -491,12 +491,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>06/02/2022</t>
+          <t>06/06/2022</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2–6–9–15–21–25</t>
+          <t>2–8–9–13–15–21</t>
         </is>
       </c>
     </row>
@@ -506,12 +506,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05/31/2022</t>
+          <t>06/03/2022</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1–6–7–8–20–25</t>
+          <t>2–3–4–15–17–24</t>
         </is>
       </c>
     </row>
@@ -521,12 +521,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05/30/2022</t>
+          <t>06/02/2022</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2–7–9–11–12–20</t>
+          <t>2–6–9–15–21–25</t>
         </is>
       </c>
     </row>
@@ -536,12 +536,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05/27/2022</t>
+          <t>05/31/2022</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>3–6–8–13–24–25</t>
+          <t>1–6–7–8–20–25</t>
         </is>
       </c>
     </row>
@@ -551,12 +551,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05/26/2022</t>
+          <t>05/30/2022</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1–2–4–7–15–18</t>
+          <t>2–7–9–11–12–20</t>
         </is>
       </c>
     </row>
@@ -566,12 +566,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05/24/2022</t>
+          <t>05/27/2022</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2–4–9–13–16–22</t>
+          <t>3–6–8–13–24–25</t>
         </is>
       </c>
     </row>
@@ -581,12 +581,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05/23/2022</t>
+          <t>05/26/2022</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>5–6–7–11–14–21</t>
+          <t>1–2–4–7–15–18</t>
         </is>
       </c>
     </row>
@@ -596,12 +596,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>05/20/2022</t>
+          <t>05/24/2022</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>4–9–15–18–23–25</t>
+          <t>2–4–9–13–16–22</t>
         </is>
       </c>
     </row>
@@ -611,12 +611,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>05/19/2022</t>
+          <t>05/23/2022</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>4–7–9–10–14–16</t>
+          <t>5–6–7–11–14–21</t>
         </is>
       </c>
     </row>
@@ -626,12 +626,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>05/17/2022</t>
+          <t>05/20/2022</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1–6–12–13–16–25</t>
+          <t>4–9–15–18–23–25</t>
         </is>
       </c>
     </row>
@@ -641,12 +641,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>05/16/2022</t>
+          <t>05/19/2022</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5–6–8–20–22–25</t>
+          <t>4–7–9–10–14–16</t>
         </is>
       </c>
     </row>
@@ -656,12 +656,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>05/13/2022</t>
+          <t>05/17/2022</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2–9–10–12–13–16</t>
+          <t>1–6–12–13–16–25</t>
         </is>
       </c>
     </row>
@@ -671,12 +671,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>05/12/2022</t>
+          <t>05/16/2022</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2–4–13–15–18–25</t>
+          <t>5–6–8–20–22–25</t>
         </is>
       </c>
     </row>
@@ -686,12 +686,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>05/10/2022</t>
+          <t>05/13/2022</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2–6–17–19–21–23</t>
+          <t>2–9–10–12–13–16</t>
         </is>
       </c>
     </row>
@@ -701,12 +701,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>05/09/2022</t>
+          <t>05/12/2022</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>3–5–10–13–18–20</t>
+          <t>2–4–13–15–18–25</t>
         </is>
       </c>
     </row>
@@ -716,12 +716,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>05/06/2022</t>
+          <t>05/10/2022</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>3–7–13–14–24–25</t>
+          <t>2–6–17–19–21–23</t>
         </is>
       </c>
     </row>
@@ -731,12 +731,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>05/05/2022</t>
+          <t>05/09/2022</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>3–5–8–17–18–25</t>
+          <t>3–5–10–13–18–20</t>
         </is>
       </c>
     </row>
@@ -746,12 +746,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>05/03/2022</t>
+          <t>05/06/2022</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1–4–13–20–22–25</t>
+          <t>3–7–13–14–24–25</t>
         </is>
       </c>
     </row>
@@ -761,12 +761,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>05/02/2022</t>
+          <t>05/05/2022</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>3–8–17–20–22–25</t>
+          <t>3–5–8–17–18–25</t>
         </is>
       </c>
     </row>
@@ -776,12 +776,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>04/29/2022</t>
+          <t>05/03/2022</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>5–6–12–17–18–23</t>
+          <t>1–4–13–20–22–25</t>
         </is>
       </c>
     </row>
@@ -791,12 +791,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>04/28/2022</t>
+          <t>05/02/2022</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1–5–10–19–20–23</t>
+          <t>3–8–17–20–22–25</t>
         </is>
       </c>
     </row>
@@ -806,12 +806,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>04/26/2022</t>
+          <t>04/29/2022</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>1–4–9–15–19–22</t>
+          <t>5–6–12–17–18–23</t>
         </is>
       </c>
     </row>
@@ -821,12 +821,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>04/25/2022</t>
+          <t>04/28/2022</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>1–2–9–18–23–24</t>
+          <t>1–5–10–19–20–23</t>
         </is>
       </c>
     </row>
@@ -836,12 +836,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>04/22/2022</t>
+          <t>04/26/2022</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>1–8–16–17–19–22</t>
+          <t>1–4–9–15–19–22</t>
         </is>
       </c>
     </row>
@@ -851,12 +851,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>04/21/2022</t>
+          <t>04/25/2022</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>3–11–19–22–23–24</t>
+          <t>1–2–9–18–23–24</t>
         </is>
       </c>
     </row>
@@ -866,12 +866,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>04/19/2022</t>
+          <t>04/22/2022</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>7–8–9–10–16–23</t>
+          <t>1–8–16–17–19–22</t>
         </is>
       </c>
     </row>
@@ -881,12 +881,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>04/18/2022</t>
+          <t>04/21/2022</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>1–18–20–21–22–23</t>
+          <t>3–11–19–22–23–24</t>
         </is>
       </c>
     </row>
@@ -896,12 +896,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>04/15/2022</t>
+          <t>04/19/2022</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2–11–14–17–22–23</t>
+          <t>7–8–9–10–16–23</t>
         </is>
       </c>
     </row>
@@ -911,12 +911,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>04/14/2022</t>
+          <t>04/18/2022</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2–3–5–11–21–23</t>
+          <t>1–18–20–21–22–23</t>
         </is>
       </c>
     </row>
@@ -926,12 +926,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>04/12/2022</t>
+          <t>04/15/2022</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>1–6–14–17–19–23</t>
+          <t>2–11–14–17–22–23</t>
         </is>
       </c>
     </row>
@@ -941,12 +941,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>04/11/2022</t>
+          <t>04/14/2022</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>12–13–14–19–21–22</t>
+          <t>2–3–5–11–21–23</t>
         </is>
       </c>
     </row>
@@ -956,12 +956,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>04/08/2022</t>
+          <t>04/12/2022</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>1–2–6–13–15–21</t>
+          <t>1–6–14–17–19–23</t>
         </is>
       </c>
     </row>
@@ -971,12 +971,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>04/07/2022</t>
+          <t>04/11/2022</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>5–10–11–12–14–15</t>
+          <t>12–13–14–19–21–22</t>
         </is>
       </c>
     </row>
@@ -986,12 +986,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>04/05/2022</t>
+          <t>04/08/2022</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2–4–6–13–14–23</t>
+          <t>1–2–6–13–15–21</t>
         </is>
       </c>
     </row>
@@ -1001,12 +1001,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>04/04/2022</t>
+          <t>04/07/2022</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>5–11–14–15–16–17</t>
+          <t>5–10–11–12–14–15</t>
         </is>
       </c>
     </row>
@@ -1016,12 +1016,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>04/01/2022</t>
+          <t>04/05/2022</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2–9–16–19–20–21</t>
+          <t>2–4–6–13–14–23</t>
         </is>
       </c>
     </row>
@@ -1031,12 +1031,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>03/31/2022</t>
+          <t>04/04/2022</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>5–11–13–14–18–22</t>
+          <t>5–11–14–15–16–17</t>
         </is>
       </c>
     </row>
@@ -1046,12 +1046,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>03/29/2022</t>
+          <t>04/01/2022</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2–4–9–16–18–19</t>
+          <t>2–9–16–19–20–21</t>
         </is>
       </c>
     </row>
@@ -1061,12 +1061,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>03/28/2022</t>
+          <t>03/31/2022</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>5–9–10–15–21–22</t>
+          <t>5–11–13–14–18–22</t>
         </is>
       </c>
     </row>
@@ -1076,12 +1076,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>03/25/2022</t>
+          <t>03/29/2022</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>6–7–16–18–23–25</t>
+          <t>2–4–9–16–18–19</t>
         </is>
       </c>
     </row>
@@ -1091,12 +1091,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>03/24/2022</t>
+          <t>03/28/2022</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>5–9–15–16–17–21</t>
+          <t>5–9–10–15–21–22</t>
         </is>
       </c>
     </row>
@@ -1106,12 +1106,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>03/22/2022</t>
+          <t>03/25/2022</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2–6–10–11–16–23</t>
+          <t>6–7–16–18–23–25</t>
         </is>
       </c>
     </row>
@@ -1121,12 +1121,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>03/21/2022</t>
+          <t>03/24/2022</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>6–9–14–16–22–23</t>
+          <t>5–9–15–16–17–21</t>
         </is>
       </c>
     </row>
@@ -1136,12 +1136,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>03/18/2022</t>
+          <t>03/22/2022</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>1–4–19–20–23–25</t>
+          <t>2–6–10–11–16–23</t>
         </is>
       </c>
     </row>
@@ -1151,12 +1151,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>03/17/2022</t>
+          <t>03/21/2022</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>1–3–4–5–8–16</t>
+          <t>6–9–14–16–22–23</t>
         </is>
       </c>
     </row>
@@ -1166,12 +1166,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>03/15/2022</t>
+          <t>03/18/2022</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>5–9–16–17–19–21</t>
+          <t>1–4–19–20–23–25</t>
         </is>
       </c>
     </row>
@@ -1181,12 +1181,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>03/14/2022</t>
+          <t>03/17/2022</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>1–4–7–13–16–24</t>
+          <t>1–3–4–5–8–16</t>
         </is>
       </c>
     </row>
@@ -1196,12 +1196,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>03/11/2022</t>
+          <t>03/15/2022</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>6–13–15–18–21–23</t>
+          <t>5–9–16–17–19–21</t>
         </is>
       </c>
     </row>
@@ -1211,12 +1211,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>03/10/2022</t>
+          <t>03/14/2022</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2–4–15–16–19–21</t>
+          <t>1–4–7–13–16–24</t>
         </is>
       </c>
     </row>
@@ -1226,12 +1226,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>03/08/2022</t>
+          <t>03/11/2022</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>1–3–4–7–10–20</t>
+          <t>6–13–15–18–21–23</t>
         </is>
       </c>
     </row>
@@ -1241,12 +1241,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>03/07/2022</t>
+          <t>03/10/2022</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>1–4–8–15–24–25</t>
+          <t>2–4–15–16–19–21</t>
         </is>
       </c>
     </row>
@@ -1256,12 +1256,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>03/04/2022</t>
+          <t>03/08/2022</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2–5–9–12–18–24</t>
+          <t>1–3–4–7–10–20</t>
         </is>
       </c>
     </row>
@@ -1271,12 +1271,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>03/03/2022</t>
+          <t>03/07/2022</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>6–7–9–12–14–22</t>
+          <t>1–4–8–15–24–25</t>
         </is>
       </c>
     </row>
@@ -1286,12 +1286,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>03/01/2022</t>
+          <t>03/04/2022</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2–7–9–14–16–20</t>
+          <t>2–5–9–12–18–24</t>
         </is>
       </c>
     </row>
@@ -1301,12 +1301,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>02/28/2022</t>
+          <t>03/03/2022</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>1–6–7–19–22–24</t>
+          <t>6–7–9–12–14–22</t>
         </is>
       </c>
     </row>
@@ -1316,12 +1316,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>02/25/2022</t>
+          <t>03/01/2022</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>3–7–9–14–15–22</t>
+          <t>2–7–9–14–16–20</t>
         </is>
       </c>
     </row>
@@ -1331,12 +1331,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>02/24/2022</t>
+          <t>02/28/2022</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>5–13–14–15–22–24</t>
+          <t>1–6–7–19–22–24</t>
         </is>
       </c>
     </row>
@@ -1346,12 +1346,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>02/22/2022</t>
+          <t>02/25/2022</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>6–9–18–20–22–23</t>
+          <t>3–7–9–14–15–22</t>
         </is>
       </c>
     </row>
@@ -1361,12 +1361,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>02/21/2022</t>
+          <t>02/24/2022</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>3–11–15–16–17–21</t>
+          <t>5–13–14–15–22–24</t>
         </is>
       </c>
     </row>
@@ -1376,12 +1376,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>02/18/2022</t>
+          <t>02/22/2022</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>1–2–10–14–22–23</t>
+          <t>6–9–18–20–22–23</t>
         </is>
       </c>
     </row>
@@ -1391,12 +1391,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>02/17/2022</t>
+          <t>02/21/2022</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>3–4–10–19–22–24</t>
+          <t>3–11–15–16–17–21</t>
         </is>
       </c>
     </row>
@@ -1406,12 +1406,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>02/15/2022</t>
+          <t>02/18/2022</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>1–9–13–15–19–20</t>
+          <t>1–2–10–14–22–23</t>
         </is>
       </c>
     </row>
@@ -1421,12 +1421,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>02/14/2022</t>
+          <t>02/17/2022</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>4–7–9–10–14–17</t>
+          <t>3–4–10–19–22–24</t>
         </is>
       </c>
     </row>
@@ -1436,12 +1436,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>02/11/2022</t>
+          <t>02/15/2022</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>4–6–8–10–12–20</t>
+          <t>1–9–13–15–19–20</t>
         </is>
       </c>
     </row>
@@ -1451,12 +1451,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>02/10/2022</t>
+          <t>02/14/2022</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>5–11–16–20–22–23</t>
+          <t>4–7–9–10–14–17</t>
         </is>
       </c>
     </row>
@@ -1466,12 +1466,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>02/08/2022</t>
+          <t>02/11/2022</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2–5–14–16–17–25</t>
+          <t>4–6–8–10–12–20</t>
         </is>
       </c>
     </row>
@@ -1481,12 +1481,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>02/07/2022</t>
+          <t>02/10/2022</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>4–7–14–16–18–23</t>
+          <t>5–11–16–20–22–23</t>
         </is>
       </c>
     </row>
@@ -1496,12 +1496,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>02/04/2022</t>
+          <t>02/08/2022</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>13–17–20–23–24–25</t>
+          <t>2–5–14–16–17–25</t>
         </is>
       </c>
     </row>
@@ -1511,12 +1511,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>02/03/2022</t>
+          <t>02/07/2022</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>6–12–14–17–22–25</t>
+          <t>4–7–14–16–18–23</t>
         </is>
       </c>
     </row>
@@ -1526,12 +1526,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>02/01/2022</t>
+          <t>02/04/2022</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>6–7–12–15–16–20</t>
+          <t>13–17–20–23–24–25</t>
         </is>
       </c>
     </row>
@@ -1541,12 +1541,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>01/31/2022</t>
+          <t>02/03/2022</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>5–7–8–9–10–22</t>
+          <t>6–12–14–17–22–25</t>
         </is>
       </c>
     </row>
@@ -1556,12 +1556,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>01/28/2022</t>
+          <t>02/01/2022</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>7–9–11–12–17–19</t>
+          <t>6–7–12–15–16–20</t>
         </is>
       </c>
     </row>
@@ -1571,12 +1571,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>01/27/2022</t>
+          <t>01/31/2022</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2–3–14–19–20–21</t>
+          <t>5–7–8–9–10–22</t>
         </is>
       </c>
     </row>
@@ -1586,12 +1586,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>01/25/2022</t>
+          <t>01/28/2022</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>3–4–5–11–17–19</t>
+          <t>7–9–11–12–17–19</t>
         </is>
       </c>
     </row>
@@ -1601,12 +1601,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>01/24/2022</t>
+          <t>01/27/2022</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>4–7–8–20–21–25</t>
+          <t>2–3–14–19–20–21</t>
         </is>
       </c>
     </row>
@@ -1616,12 +1616,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>01/21/2022</t>
+          <t>01/25/2022</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>8–11–14–15–18–24</t>
+          <t>3–4–5–11–17–19</t>
         </is>
       </c>
     </row>
@@ -1631,12 +1631,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>01/20/2022</t>
+          <t>01/24/2022</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2–15–19–20–22–24</t>
+          <t>4–7–8–20–21–25</t>
         </is>
       </c>
     </row>
@@ -1646,12 +1646,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>01/18/2022</t>
+          <t>01/21/2022</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>3–5–16–17–18–21</t>
+          <t>8–11–14–15–18–24</t>
         </is>
       </c>
     </row>
@@ -1661,12 +1661,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>01/17/2022</t>
+          <t>01/20/2022</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>5–8–16–18–20–22</t>
+          <t>2–15–19–20–22–24</t>
         </is>
       </c>
     </row>
@@ -1676,12 +1676,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>01/14/2022</t>
+          <t>01/18/2022</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2–5–8–9–10–13</t>
+          <t>3–5–16–17–18–21</t>
         </is>
       </c>
     </row>
@@ -1691,12 +1691,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>01/13/2022</t>
+          <t>01/17/2022</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2–6–8–11–18–21</t>
+          <t>5–8–16–18–20–22</t>
         </is>
       </c>
     </row>
@@ -1706,12 +1706,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>01/11/2022</t>
+          <t>01/14/2022</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>7–8–9–15–19–23</t>
+          <t>2–5–8–9–10–13</t>
         </is>
       </c>
     </row>
@@ -1721,12 +1721,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>01/10/2022</t>
+          <t>01/13/2022</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>10–13–14–19–22–23</t>
+          <t>2–6–8–11–18–21</t>
         </is>
       </c>
     </row>
@@ -1736,12 +1736,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>01/07/2022</t>
+          <t>01/11/2022</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>4–8–21–23–24–25</t>
+          <t>7–8–9–15–19–23</t>
         </is>
       </c>
     </row>
@@ -1751,12 +1751,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>01/06/2022</t>
+          <t>01/10/2022</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>7–9–10–17–18–23</t>
+          <t>10–13–14–19–22–23</t>
         </is>
       </c>
     </row>
@@ -1766,12 +1766,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>01/04/2022</t>
+          <t>01/07/2022</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>4–7–14–15–24–25</t>
+          <t>4–8–21–23–24–25</t>
         </is>
       </c>
     </row>
@@ -1781,12 +1781,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>01/03/2022</t>
+          <t>01/06/2022</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>6–10–17–18–19–21</t>
+          <t>7–9–10–17–18–23</t>
         </is>
       </c>
     </row>
@@ -1796,12 +1796,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>12/31/2021</t>
+          <t>01/04/2022</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>11–17–20–22–23–24</t>
+          <t>4–7–14–15–24–25</t>
         </is>
       </c>
     </row>
@@ -1811,12 +1811,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>12/30/2021</t>
+          <t>01/03/2022</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>1–8–9–13–20–25</t>
+          <t>6–10–17–18–19–21</t>
         </is>
       </c>
     </row>
@@ -1826,12 +1826,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>12/28/2021</t>
+          <t>12/31/2021</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>4–9–11–15–16–25</t>
+          <t>11–17–20–22–23–24</t>
         </is>
       </c>
     </row>
@@ -1841,12 +1841,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>12/27/2021</t>
+          <t>12/30/2021</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>3–4–10–14–19–25</t>
+          <t>1–8–9–13–20–25</t>
         </is>
       </c>
     </row>
@@ -1856,12 +1856,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>12/24/2021</t>
+          <t>12/28/2021</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>4–6–13–17–21–22</t>
+          <t>4–9–11–15–16–25</t>
         </is>
       </c>
     </row>
@@ -1871,12 +1871,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>12/23/2021</t>
+          <t>12/27/2021</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>1–2–3–15–20–23</t>
+          <t>3–4–10–14–19–25</t>
         </is>
       </c>
     </row>
@@ -1886,12 +1886,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>12/21/2021</t>
+          <t>12/24/2021</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>6–9–11–12–14–25</t>
+          <t>4–6–13–17–21–22</t>
         </is>
       </c>
     </row>
@@ -1901,12 +1901,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>12/20/2021</t>
+          <t>12/23/2021</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>7–8–9–22–23–24</t>
+          <t>1–2–3–15–20–23</t>
         </is>
       </c>
     </row>
@@ -1916,12 +1916,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>12/17/2021</t>
+          <t>12/21/2021</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>3–9–15–16–18–22</t>
+          <t>6–9–11–12–14–25</t>
         </is>
       </c>
     </row>
@@ -1931,12 +1931,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>12/16/2021</t>
+          <t>12/20/2021</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2–3–11–13–24–25</t>
+          <t>7–8–9–22–23–24</t>
         </is>
       </c>
     </row>
@@ -1946,12 +1946,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>12/14/2021</t>
+          <t>12/17/2021</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2–7–9–17–23–24</t>
+          <t>3–9–15–16–18–22</t>
         </is>
       </c>
     </row>
@@ -1961,12 +1961,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>12/13/2021</t>
+          <t>12/16/2021</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2–6–15–16–23–24</t>
+          <t>2–3–11–13–24–25</t>
         </is>
       </c>
     </row>
@@ -1976,12 +1976,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>12/10/2021</t>
+          <t>12/14/2021</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>3–6–9–10–14–21</t>
+          <t>2–7–9–17–23–24</t>
         </is>
       </c>
     </row>
@@ -1991,12 +1991,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>12/09/2021</t>
+          <t>12/13/2021</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2–12–14–15–19–21</t>
+          <t>2–6–15–16–23–24</t>
         </is>
       </c>
     </row>
@@ -2006,12 +2006,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>12/07/2021</t>
+          <t>12/10/2021</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>3–5–8–9–16–25</t>
+          <t>3–6–9–10–14–21</t>
         </is>
       </c>
     </row>
@@ -2021,12 +2021,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>12/06/2021</t>
+          <t>12/09/2021</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>3–5–8–12–15–19</t>
+          <t>2–12–14–15–19–21</t>
         </is>
       </c>
     </row>
@@ -2036,12 +2036,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>12/03/2021</t>
+          <t>12/07/2021</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>10–13–14–15–21–24</t>
+          <t>3–5–8–9–16–25</t>
         </is>
       </c>
     </row>
@@ -2051,12 +2051,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>12/02/2021</t>
+          <t>12/06/2021</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2–7–8–11–22–24</t>
+          <t>3–5–8–12–15–19</t>
         </is>
       </c>
     </row>
@@ -2066,12 +2066,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>11/30/2021</t>
+          <t>12/03/2021</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>12–14–20–23–24–25</t>
+          <t>10–13–14–15–21–24</t>
         </is>
       </c>
     </row>
@@ -2081,12 +2081,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>11/29/2021</t>
+          <t>12/02/2021</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>4–8–10–13–20–21</t>
+          <t>2–7–8–11–22–24</t>
         </is>
       </c>
     </row>
@@ -2096,12 +2096,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>11/26/2021</t>
+          <t>11/30/2021</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>3–7–14–17–24–25</t>
+          <t>12–14–20–23–24–25</t>
         </is>
       </c>
     </row>
@@ -2111,12 +2111,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>11/25/2021</t>
+          <t>11/29/2021</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2–11–16–18–20–21</t>
+          <t>4–8–10–13–20–21</t>
         </is>
       </c>
     </row>
@@ -2126,12 +2126,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>11/23/2021</t>
+          <t>11/26/2021</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2–10–11–12–14–19</t>
+          <t>3–7–14–17–24–25</t>
         </is>
       </c>
     </row>
@@ -2141,12 +2141,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>11/22/2021</t>
+          <t>11/25/2021</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>5–10–12–16–20–25</t>
+          <t>2–11–16–18–20–21</t>
         </is>
       </c>
     </row>
@@ -2156,12 +2156,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>11/19/2021</t>
+          <t>11/23/2021</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>12–16–19–20–21–24</t>
+          <t>2–10–11–12–14–19</t>
         </is>
       </c>
     </row>
@@ -2171,12 +2171,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>11/18/2021</t>
+          <t>11/22/2021</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>1–4–17–18–20–23</t>
+          <t>5–10–12–16–20–25</t>
         </is>
       </c>
     </row>
@@ -2186,12 +2186,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>11/16/2021</t>
+          <t>11/19/2021</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>5–8–10–11–16–23</t>
+          <t>12–16–19–20–21–24</t>
         </is>
       </c>
     </row>
@@ -2201,12 +2201,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>11/15/2021</t>
+          <t>11/18/2021</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2–6–10–11–15–18</t>
+          <t>1–4–17–18–20–23</t>
         </is>
       </c>
     </row>
@@ -2216,12 +2216,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>11/12/2021</t>
+          <t>11/16/2021</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>1–13–14–15–22–25</t>
+          <t>5–8–10–11–16–23</t>
         </is>
       </c>
     </row>
@@ -2231,12 +2231,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>11/11/2021</t>
+          <t>11/15/2021</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>2–3–5–14–21–22</t>
+          <t>2–6–10–11–15–18</t>
         </is>
       </c>
     </row>
@@ -2246,12 +2246,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>11/09/2021</t>
+          <t>11/12/2021</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2–4–10–13–16–23</t>
+          <t>1–13–14–15–22–25</t>
         </is>
       </c>
     </row>
@@ -2261,12 +2261,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>11/08/2021</t>
+          <t>11/11/2021</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>1–2–8–10–13–24</t>
+          <t>2–3–5–14–21–22</t>
         </is>
       </c>
     </row>
@@ -2276,12 +2276,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>11/05/2021</t>
+          <t>11/09/2021</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>4–11–12–18–19–25</t>
+          <t>2–4–10–13–16–23</t>
         </is>
       </c>
     </row>
@@ -2291,12 +2291,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>11/04/2021</t>
+          <t>11/08/2021</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>10–15–19–21–24–25</t>
+          <t>1–2–8–10–13–24</t>
         </is>
       </c>
     </row>
@@ -2306,12 +2306,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>11/02/2021</t>
+          <t>11/05/2021</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>3–4–9–16–17–18</t>
+          <t>4–11–12–18–19–25</t>
         </is>
       </c>
     </row>
@@ -2321,12 +2321,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>11/01/2021</t>
+          <t>11/04/2021</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>5–6–14–15–18–20</t>
+          <t>10–15–19–21–24–25</t>
         </is>
       </c>
     </row>
@@ -2336,12 +2336,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>10/29/2021</t>
+          <t>11/02/2021</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2–3–8–9–13–15</t>
+          <t>3–4–9–16–17–18</t>
         </is>
       </c>
     </row>
@@ -2351,12 +2351,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>10/28/2021</t>
+          <t>11/01/2021</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>7–15–19–20–23–24</t>
+          <t>5–6–14–15–18–20</t>
         </is>
       </c>
     </row>
@@ -2366,12 +2366,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>10/26/2021</t>
+          <t>10/29/2021</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>3–4–14–16–17–25</t>
+          <t>2–3–8–9–13–15</t>
         </is>
       </c>
     </row>
@@ -2381,12 +2381,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>10/25/2021</t>
+          <t>10/28/2021</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>9–12–17–19–20–24</t>
+          <t>7–15–19–20–23–24</t>
         </is>
       </c>
     </row>
@@ -2396,12 +2396,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>10/22/2021</t>
+          <t>10/26/2021</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2–5–6–18–20–23</t>
+          <t>3–4–14–16–17–25</t>
         </is>
       </c>
     </row>
@@ -2411,12 +2411,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>10/21/2021</t>
+          <t>10/25/2021</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>5–8–9–13–22–24</t>
+          <t>9–12–17–19–20–24</t>
         </is>
       </c>
     </row>
@@ -2426,12 +2426,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>10/19/2021</t>
+          <t>10/22/2021</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>8–9–11–15–19–25</t>
+          <t>2–5–6–18–20–23</t>
         </is>
       </c>
     </row>
@@ -2441,12 +2441,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>10/18/2021</t>
+          <t>10/21/2021</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>3–4–8–10–12–20</t>
+          <t>5–8–9–13–22–24</t>
         </is>
       </c>
     </row>
@@ -2456,12 +2456,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>10/15/2021</t>
+          <t>10/19/2021</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>1–3–4–8–19–21</t>
+          <t>8–9–11–15–19–25</t>
         </is>
       </c>
     </row>
@@ -2471,12 +2471,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>10/14/2021</t>
+          <t>10/18/2021</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2–5–8–15–16–23</t>
+          <t>3–4–8–10–12–20</t>
         </is>
       </c>
     </row>
@@ -2486,12 +2486,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>10/12/2021</t>
+          <t>10/15/2021</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>5–6–13–14–24–25</t>
+          <t>1–3–4–8–19–21</t>
         </is>
       </c>
     </row>
@@ -2501,12 +2501,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>10/11/2021</t>
+          <t>10/14/2021</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>1–2–3–5–21–23</t>
+          <t>2–5–8–15–16–23</t>
         </is>
       </c>
     </row>
@@ -2516,12 +2516,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>10/08/2021</t>
+          <t>10/12/2021</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>10–11–13–17–20–22</t>
+          <t>5–6–13–14–24–25</t>
         </is>
       </c>
     </row>
@@ -2531,12 +2531,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>10/07/2021</t>
+          <t>10/11/2021</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>3–5–8–16–19–23</t>
+          <t>1–2–3–5–21–23</t>
         </is>
       </c>
     </row>
@@ -2546,12 +2546,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>10/05/2021</t>
+          <t>10/08/2021</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>7–9–13–15–18–23</t>
+          <t>10–11–13–17–20–22</t>
         </is>
       </c>
     </row>
@@ -2561,12 +2561,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>10/04/2021</t>
+          <t>10/07/2021</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>8–9–11–18–20–23</t>
+          <t>3–5–8–16–19–23</t>
         </is>
       </c>
     </row>
@@ -2576,12 +2576,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>10/01/2021</t>
+          <t>10/05/2021</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2–3–5–7–11–18</t>
+          <t>7–9–13–15–18–23</t>
         </is>
       </c>
     </row>
@@ -2591,12 +2591,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>09/30/2021</t>
+          <t>10/04/2021</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>5–16–18–20–22–24</t>
+          <t>8–9–11–18–20–23</t>
         </is>
       </c>
     </row>
@@ -2606,12 +2606,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>09/28/2021</t>
+          <t>10/01/2021</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>1–9–11–12–18–22</t>
+          <t>2–3–5–7–11–18</t>
         </is>
       </c>
     </row>
@@ -2621,12 +2621,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>09/27/2021</t>
+          <t>09/30/2021</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>4–5–6–10–14–22</t>
+          <t>5–16–18–20–22–24</t>
         </is>
       </c>
     </row>
@@ -2636,12 +2636,12 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>09/24/2021</t>
+          <t>09/28/2021</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>4–11–15–16–22–25</t>
+          <t>1–9–11–12–18–22</t>
         </is>
       </c>
     </row>
@@ -2651,12 +2651,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>09/23/2021</t>
+          <t>09/27/2021</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>4–9–13–15–17–18</t>
+          <t>4–5–6–10–14–22</t>
         </is>
       </c>
     </row>
@@ -2666,12 +2666,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>09/21/2021</t>
+          <t>09/24/2021</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>1–13–14–21–22–24</t>
+          <t>4–11–15–16–22–25</t>
         </is>
       </c>
     </row>
@@ -2681,12 +2681,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>09/20/2021</t>
+          <t>09/23/2021</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>1–13–17–18–20–22</t>
+          <t>4–9–13–15–17–18</t>
         </is>
       </c>
     </row>
@@ -2696,12 +2696,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>09/17/2021</t>
+          <t>09/21/2021</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2–6–8–9–11–12</t>
+          <t>1–13–14–21–22–24</t>
         </is>
       </c>
     </row>
@@ -2711,12 +2711,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>09/16/2021</t>
+          <t>09/20/2021</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2–11–12–14–17–19</t>
+          <t>1–13–17–18–20–22</t>
         </is>
       </c>
     </row>
@@ -2726,12 +2726,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>09/14/2021</t>
+          <t>09/17/2021</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>4–11–18–19–20–23</t>
+          <t>2–6–8–9–11–12</t>
         </is>
       </c>
     </row>
@@ -2741,12 +2741,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>09/13/2021</t>
+          <t>09/16/2021</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>1–8–11–12–13–18</t>
+          <t>2–11–12–14–17–19</t>
         </is>
       </c>
     </row>
@@ -2756,12 +2756,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>09/10/2021</t>
+          <t>09/14/2021</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>3–4–6–8–11–16</t>
+          <t>4–11–18–19–20–23</t>
         </is>
       </c>
     </row>
@@ -2771,12 +2771,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>09/09/2021</t>
+          <t>09/13/2021</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>1–14–15–20–21–25</t>
+          <t>1–8–11–12–13–18</t>
         </is>
       </c>
     </row>
@@ -2786,12 +2786,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>09/07/2021</t>
+          <t>09/10/2021</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>5–7–8–9–18–21</t>
+          <t>3–4–6–8–11–16</t>
         </is>
       </c>
     </row>
@@ -2801,12 +2801,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>09/06/2021</t>
+          <t>09/09/2021</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>6–7–9–16–21–22</t>
+          <t>1–14–15–20–21–25</t>
         </is>
       </c>
     </row>
@@ -2816,12 +2816,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>09/03/2021</t>
+          <t>09/07/2021</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>1–3–11–21–22–24</t>
+          <t>5–7–8–9–18–21</t>
         </is>
       </c>
     </row>
@@ -2831,12 +2831,12 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>09/02/2021</t>
+          <t>09/06/2021</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>1–2–4–10–11–24</t>
+          <t>6–7–9–16–21–22</t>
         </is>
       </c>
     </row>
@@ -2846,12 +2846,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>08/31/2021</t>
+          <t>09/03/2021</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>1–8–9–15–19–21</t>
+          <t>1–3–11–21–22–24</t>
         </is>
       </c>
     </row>
@@ -2861,12 +2861,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>08/30/2021</t>
+          <t>09/02/2021</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>5–10–19–20–21–25</t>
+          <t>1–2–4–10–11–24</t>
         </is>
       </c>
     </row>
@@ -2876,12 +2876,12 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>08/27/2021</t>
+          <t>08/31/2021</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>1–10–15–17–18–21</t>
+          <t>1–8–9–15–19–21</t>
         </is>
       </c>
     </row>
@@ -2891,12 +2891,12 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>08/26/2021</t>
+          <t>08/30/2021</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>6–14–18–19–23–25</t>
+          <t>5–10–19–20–21–25</t>
         </is>
       </c>
     </row>
@@ -2906,12 +2906,12 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>08/24/2021</t>
+          <t>08/27/2021</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2–3–6–20–21–23</t>
+          <t>1–10–15–17–18–21</t>
         </is>
       </c>
     </row>
@@ -2921,12 +2921,12 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>08/23/2021</t>
+          <t>08/26/2021</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>9–11–12–14–18–23</t>
+          <t>6–14–18–19–23–25</t>
         </is>
       </c>
     </row>
@@ -2936,12 +2936,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>08/20/2021</t>
+          <t>08/24/2021</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>5–8–17–19–20–24</t>
+          <t>2–3–6–20–21–23</t>
         </is>
       </c>
     </row>
@@ -2951,12 +2951,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>08/19/2021</t>
+          <t>08/23/2021</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2–3–6–8–12–21</t>
+          <t>9–11–12–14–18–23</t>
         </is>
       </c>
     </row>
@@ -2966,12 +2966,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>08/17/2021</t>
+          <t>08/20/2021</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>7–12–15–16–20–25</t>
+          <t>5–8–17–19–20–24</t>
         </is>
       </c>
     </row>
@@ -2981,12 +2981,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>08/16/2021</t>
+          <t>08/19/2021</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>1–3–5–8–9–15</t>
+          <t>2–3–6–8–12–21</t>
         </is>
       </c>
     </row>
@@ -2996,12 +2996,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>08/13/2021</t>
+          <t>08/17/2021</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>1–5–10–14–18–24</t>
+          <t>7–12–15–16–20–25</t>
         </is>
       </c>
     </row>
@@ -3011,12 +3011,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>08/12/2021</t>
+          <t>08/16/2021</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>4–7–13–17–21–22</t>
+          <t>1–3–5–8–9–15</t>
         </is>
       </c>
     </row>
@@ -3026,12 +3026,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>08/10/2021</t>
+          <t>08/13/2021</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>4–6–9–10–15–24</t>
+          <t>1–5–10–14–18–24</t>
         </is>
       </c>
     </row>
@@ -3041,12 +3041,12 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>08/09/2021</t>
+          <t>08/12/2021</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>1–2–6–13–18–25</t>
+          <t>4–7–13–17–21–22</t>
         </is>
       </c>
     </row>
@@ -3056,12 +3056,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>08/06/2021</t>
+          <t>08/10/2021</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>5–8–9–14–23–24</t>
+          <t>4–6–9–10–15–24</t>
         </is>
       </c>
     </row>
@@ -3071,12 +3071,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>08/05/2021</t>
+          <t>08/09/2021</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2–5–6–12–14–18</t>
+          <t>1–2–6–13–18–25</t>
         </is>
       </c>
     </row>
@@ -3086,12 +3086,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>08/03/2021</t>
+          <t>08/06/2021</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2–7–17–22–24–25</t>
+          <t>5–8–9–14–23–24</t>
         </is>
       </c>
     </row>
@@ -3101,12 +3101,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>08/02/2021</t>
+          <t>08/05/2021</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>7–12–13–18–22–24</t>
+          <t>2–5–6–12–14–18</t>
         </is>
       </c>
     </row>
@@ -3116,12 +3116,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>07/30/2021</t>
+          <t>08/03/2021</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>3–4–13–22–24–25</t>
+          <t>2–7–17–22–24–25</t>
         </is>
       </c>
     </row>
@@ -3131,12 +3131,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>07/29/2021</t>
+          <t>08/02/2021</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>5–7–12–17–19–24</t>
+          <t>7–12–13–18–22–24</t>
         </is>
       </c>
     </row>
@@ -3146,12 +3146,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>07/27/2021</t>
+          <t>07/30/2021</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>1–4–16–17–18–21</t>
+          <t>3–4–13–22–24–25</t>
         </is>
       </c>
     </row>
@@ -3161,12 +3161,12 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>07/26/2021</t>
+          <t>07/29/2021</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>3–14–19–21–23–24</t>
+          <t>5–7–12–17–19–24</t>
         </is>
       </c>
     </row>
@@ -3176,12 +3176,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>07/23/2021</t>
+          <t>07/27/2021</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>9–12–14–16–22–25</t>
+          <t>1–4–16–17–18–21</t>
         </is>
       </c>
     </row>
@@ -3191,12 +3191,12 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>07/22/2021</t>
+          <t>07/26/2021</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2–5–6–15–16–20</t>
+          <t>3–14–19–21–23–24</t>
         </is>
       </c>
     </row>
@@ -3206,12 +3206,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>07/20/2021</t>
+          <t>07/23/2021</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>4–7–12–15–20–21</t>
+          <t>9–12–14–16–22–25</t>
         </is>
       </c>
     </row>
@@ -3221,12 +3221,12 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>07/19/2021</t>
+          <t>07/22/2021</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2–5–9–10–18–22</t>
+          <t>2–5–6–15–16–20</t>
         </is>
       </c>
     </row>
@@ -3236,12 +3236,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>07/16/2021</t>
+          <t>07/20/2021</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>4–8–10–11–12–21</t>
+          <t>4–7–12–15–20–21</t>
         </is>
       </c>
     </row>
@@ -3251,12 +3251,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>07/15/2021</t>
+          <t>07/19/2021</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>1–6–9–11–17–22</t>
+          <t>2–5–9–10–18–22</t>
         </is>
       </c>
     </row>
@@ -3266,12 +3266,12 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>07/13/2021</t>
+          <t>07/16/2021</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>4–11–14–15–17–18</t>
+          <t>4–8–10–11–12–21</t>
         </is>
       </c>
     </row>
@@ -3281,12 +3281,12 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>07/12/2021</t>
+          <t>07/15/2021</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>1–4–5–7–8–22</t>
+          <t>1–6–9–11–17–22</t>
         </is>
       </c>
     </row>
@@ -3296,12 +3296,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>07/09/2021</t>
+          <t>07/13/2021</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>7–13–14–16–21–22</t>
+          <t>4–11–14–15–17–18</t>
         </is>
       </c>
     </row>
@@ -3311,12 +3311,12 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>07/08/2021</t>
+          <t>07/12/2021</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>5–8–9–13–14–16</t>
+          <t>1–4–5–7–8–22</t>
         </is>
       </c>
     </row>
@@ -3326,12 +3326,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>07/06/2021</t>
+          <t>07/09/2021</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>1–18–20–21–22–25</t>
+          <t>7–13–14–16–21–22</t>
         </is>
       </c>
     </row>
@@ -3341,12 +3341,12 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>07/05/2021</t>
+          <t>07/08/2021</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>3–7–11–12–13–23</t>
+          <t>5–8–9–13–14–16</t>
         </is>
       </c>
     </row>
@@ -3356,12 +3356,12 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>07/02/2021</t>
+          <t>07/06/2021</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>1–4–5–8–14–20</t>
+          <t>1–18–20–21–22–25</t>
         </is>
       </c>
     </row>
@@ -3371,12 +3371,12 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>07/01/2021</t>
+          <t>07/05/2021</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>6–9–11–14–16–19</t>
+          <t>3–7–11–12–13–23</t>
         </is>
       </c>
     </row>
@@ -3386,12 +3386,12 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>06/29/2021</t>
+          <t>07/02/2021</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>1–5–9–10–16–20</t>
+          <t>1–4–5–8–14–20</t>
         </is>
       </c>
     </row>
@@ -3401,12 +3401,12 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>06/28/2021</t>
+          <t>07/01/2021</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>4–14–18–20–21–22</t>
+          <t>6–9–11–14–16–19</t>
         </is>
       </c>
     </row>
@@ -3416,12 +3416,12 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>06/25/2021</t>
+          <t>06/29/2021</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>1–3–4–7–11–18</t>
+          <t>1–5–9–10–16–20</t>
         </is>
       </c>
     </row>
@@ -3431,12 +3431,12 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>06/24/2021</t>
+          <t>06/28/2021</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>1–5–9–11–20–22</t>
+          <t>4–14–18–20–21–22</t>
         </is>
       </c>
     </row>
@@ -3446,12 +3446,12 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>06/22/2021</t>
+          <t>06/25/2021</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>7–9–12–18–21–23</t>
+          <t>1–3–4–7–11–18</t>
         </is>
       </c>
     </row>
@@ -3461,12 +3461,12 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>06/21/2021</t>
+          <t>06/24/2021</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>7–11–17–18–23–24</t>
+          <t>1–5–9–11–20–22</t>
         </is>
       </c>
     </row>
@@ -3476,12 +3476,12 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>06/18/2021</t>
+          <t>06/22/2021</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>2–7–11–17–18–25</t>
+          <t>7–9–12–18–21–23</t>
         </is>
       </c>
     </row>
@@ -3491,12 +3491,12 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>06/17/2021</t>
+          <t>06/21/2021</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>3–12–17–19–24–25</t>
+          <t>7–11–17–18–23–24</t>
         </is>
       </c>
     </row>
@@ -3506,12 +3506,12 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>06/15/2021</t>
+          <t>06/18/2021</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>3–5–12–16–18–23</t>
+          <t>2–7–11–17–18–25</t>
         </is>
       </c>
     </row>
@@ -3521,12 +3521,12 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>06/14/2021</t>
+          <t>06/17/2021</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>1–5–11–12–22–23</t>
+          <t>3–12–17–19–24–25</t>
         </is>
       </c>
     </row>
@@ -3536,12 +3536,12 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>06/11/2021</t>
+          <t>06/15/2021</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>2–5–10–11–24–25</t>
+          <t>3–5–12–16–18–23</t>
         </is>
       </c>
     </row>
@@ -3551,12 +3551,12 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>06/10/2021</t>
+          <t>06/14/2021</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>7–10–13–14–18–21</t>
+          <t>1–5–11–12–22–23</t>
         </is>
       </c>
     </row>
@@ -3566,12 +3566,12 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>06/08/2021</t>
+          <t>06/11/2021</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>8–9–15–16–23–25</t>
+          <t>2–5–10–11–24–25</t>
         </is>
       </c>
     </row>

</xml_diff>